<commit_message>
PLS FINAL 1 EVER (it wasnt)
</commit_message>
<xml_diff>
--- a/0. data_raw_excel/COVER Data/2013-14-nhs-immu-stat-eng-tab-exc.xlsx
+++ b/0. data_raw_excel/COVER Data/2013-14-nhs-immu-stat-eng-tab-exc.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://stummuac-my.sharepoint.com/personal/25943553_stu_mmu_ac_uk/Documents/03 DISSERTATION/GITHUB/0. data_raw_excel/COVER Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="11" documentId="11_4808CF6E242D889673B717D637D25F605D6AF9A7" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{871A9E03-16E3-4989-A1F6-3F8DFBAF0E62}"/>
+  <xr:revisionPtr revIDLastSave="27" documentId="11_4808CF6E242D889673B717D637D25F605D6AF9A7" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{07539151-2AB2-4211-8833-C658C3AA6A38}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="0" yWindow="135" windowWidth="24300" windowHeight="15375" tabRatio="882" firstSheet="10" activeTab="24" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11025" yWindow="4245" windowWidth="17775" windowHeight="11505" tabRatio="882" firstSheet="10" activeTab="17" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Contents-Data Summary" sheetId="20" r:id="rId1"/>
@@ -86,7 +86,6 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="22">'Table 14a'!$1:$10</definedName>
   </definedNames>
   <calcPr calcId="145621"/>
-  <fileRecoveryPr repairLoad="1"/>
 </workbook>
 </file>
 
@@ -5644,23 +5643,11 @@
     <xf numFmtId="3" fontId="26" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="52" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="51" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -5723,6 +5710,9 @@
     <xf numFmtId="1" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="1" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -5759,6 +5749,12 @@
     <xf numFmtId="49" fontId="40" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="1" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -5768,7 +5764,10 @@
     <xf numFmtId="1" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -5776,6 +5775,12 @@
     </xf>
     <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="48" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -5794,12 +5799,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="52" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="51" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="43">
@@ -6808,20 +6807,20 @@
       <c r="B5" s="22"/>
       <c r="C5" s="22"/>
       <c r="D5" s="28"/>
-      <c r="F5" s="365" t="s">
+      <c r="F5" s="404" t="s">
         <v>548</v>
       </c>
-      <c r="G5" s="365"/>
+      <c r="G5" s="404"/>
     </row>
     <row r="6" spans="1:7">
       <c r="A6" s="33"/>
       <c r="B6" s="22"/>
       <c r="C6" s="22"/>
       <c r="D6" s="28"/>
-      <c r="F6" s="365" t="s">
+      <c r="F6" s="404" t="s">
         <v>549</v>
       </c>
-      <c r="G6" s="365"/>
+      <c r="G6" s="404"/>
     </row>
     <row r="7" spans="1:7">
       <c r="A7" s="33"/>
@@ -10160,16 +10159,16 @@
       <c r="G197" s="39"/>
     </row>
     <row r="198" spans="1:8" ht="31.5" customHeight="1">
-      <c r="A198" s="368" t="s">
+      <c r="A198" s="386" t="s">
         <v>745</v>
       </c>
-      <c r="B198" s="368"/>
-      <c r="C198" s="368"/>
-      <c r="D198" s="368"/>
-      <c r="E198" s="368"/>
-      <c r="F198" s="368"/>
-      <c r="G198" s="368"/>
-      <c r="H198" s="368"/>
+      <c r="B198" s="386"/>
+      <c r="C198" s="386"/>
+      <c r="D198" s="386"/>
+      <c r="E198" s="386"/>
+      <c r="F198" s="386"/>
+      <c r="G198" s="386"/>
+      <c r="H198" s="386"/>
     </row>
     <row r="199" spans="1:8">
       <c r="B199" s="22"/>
@@ -10180,52 +10179,52 @@
       <c r="G199" s="29"/>
     </row>
     <row r="200" spans="1:8" s="167" customFormat="1" ht="18.75" customHeight="1">
-      <c r="A200" s="364" t="s">
+      <c r="A200" s="405" t="s">
         <v>648</v>
       </c>
-      <c r="B200" s="364"/>
-      <c r="C200" s="364"/>
-      <c r="D200" s="364"/>
-      <c r="E200" s="364"/>
-      <c r="F200" s="364"/>
-      <c r="G200" s="364"/>
-      <c r="H200" s="364"/>
+      <c r="B200" s="405"/>
+      <c r="C200" s="405"/>
+      <c r="D200" s="405"/>
+      <c r="E200" s="405"/>
+      <c r="F200" s="405"/>
+      <c r="G200" s="405"/>
+      <c r="H200" s="405"/>
     </row>
     <row r="201" spans="1:8" s="167" customFormat="1" ht="35.1" customHeight="1">
-      <c r="A201" s="364" t="s">
+      <c r="A201" s="405" t="s">
         <v>653</v>
       </c>
-      <c r="B201" s="364"/>
-      <c r="C201" s="364"/>
-      <c r="D201" s="364"/>
-      <c r="E201" s="364"/>
-      <c r="F201" s="364"/>
-      <c r="G201" s="364"/>
-      <c r="H201" s="364"/>
+      <c r="B201" s="405"/>
+      <c r="C201" s="405"/>
+      <c r="D201" s="405"/>
+      <c r="E201" s="405"/>
+      <c r="F201" s="405"/>
+      <c r="G201" s="405"/>
+      <c r="H201" s="405"/>
     </row>
     <row r="202" spans="1:8" s="167" customFormat="1" ht="18.75" customHeight="1">
-      <c r="A202" s="364" t="s">
+      <c r="A202" s="405" t="s">
         <v>652</v>
       </c>
-      <c r="B202" s="364"/>
-      <c r="C202" s="364"/>
-      <c r="D202" s="364"/>
-      <c r="E202" s="364"/>
-      <c r="F202" s="364"/>
-      <c r="G202" s="364"/>
-      <c r="H202" s="364"/>
+      <c r="B202" s="405"/>
+      <c r="C202" s="405"/>
+      <c r="D202" s="405"/>
+      <c r="E202" s="405"/>
+      <c r="F202" s="405"/>
+      <c r="G202" s="405"/>
+      <c r="H202" s="405"/>
     </row>
     <row r="203" spans="1:8" s="167" customFormat="1" ht="18.75" customHeight="1">
-      <c r="A203" s="367" t="s">
+      <c r="A203" s="399" t="s">
         <v>689</v>
       </c>
-      <c r="B203" s="367"/>
-      <c r="C203" s="367"/>
-      <c r="D203" s="367"/>
-      <c r="E203" s="367"/>
-      <c r="F203" s="367"/>
-      <c r="G203" s="367"/>
-      <c r="H203" s="367"/>
+      <c r="B203" s="399"/>
+      <c r="C203" s="399"/>
+      <c r="D203" s="399"/>
+      <c r="E203" s="399"/>
+      <c r="F203" s="399"/>
+      <c r="G203" s="399"/>
+      <c r="H203" s="399"/>
     </row>
     <row r="204" spans="1:8" ht="18.75">
       <c r="A204" s="22" t="s">
@@ -10239,16 +10238,16 @@
       <c r="G204" s="29"/>
     </row>
     <row r="205" spans="1:8" s="167" customFormat="1" ht="18.75" customHeight="1">
-      <c r="A205" s="364" t="s">
+      <c r="A205" s="405" t="s">
         <v>656</v>
       </c>
-      <c r="B205" s="364"/>
-      <c r="C205" s="364"/>
-      <c r="D205" s="364"/>
-      <c r="E205" s="364"/>
-      <c r="F205" s="364"/>
-      <c r="G205" s="364"/>
-      <c r="H205" s="364"/>
+      <c r="B205" s="405"/>
+      <c r="C205" s="405"/>
+      <c r="D205" s="405"/>
+      <c r="E205" s="405"/>
+      <c r="F205" s="405"/>
+      <c r="G205" s="405"/>
+      <c r="H205" s="405"/>
     </row>
     <row r="206" spans="1:8" ht="18.75">
       <c r="A206" s="22" t="s">
@@ -10262,16 +10261,16 @@
       <c r="G206" s="29"/>
     </row>
     <row r="207" spans="1:8" s="167" customFormat="1" ht="18.75" customHeight="1">
-      <c r="A207" s="364" t="s">
+      <c r="A207" s="405" t="s">
         <v>681</v>
       </c>
-      <c r="B207" s="364"/>
-      <c r="C207" s="364"/>
-      <c r="D207" s="364"/>
-      <c r="E207" s="364"/>
-      <c r="F207" s="364"/>
-      <c r="G207" s="364"/>
-      <c r="H207" s="364"/>
+      <c r="B207" s="405"/>
+      <c r="C207" s="405"/>
+      <c r="D207" s="405"/>
+      <c r="E207" s="405"/>
+      <c r="F207" s="405"/>
+      <c r="G207" s="405"/>
+      <c r="H207" s="405"/>
     </row>
     <row r="208" spans="1:8" ht="18.75">
       <c r="A208" s="22" t="s">
@@ -10420,20 +10419,20 @@
       <c r="B5" s="22"/>
       <c r="C5" s="22"/>
       <c r="D5" s="28"/>
-      <c r="F5" s="365" t="s">
+      <c r="F5" s="404" t="s">
         <v>547</v>
       </c>
-      <c r="G5" s="365"/>
+      <c r="G5" s="404"/>
     </row>
     <row r="6" spans="1:7" ht="15.75" customHeight="1">
       <c r="A6" s="33"/>
       <c r="B6" s="22"/>
       <c r="C6" s="22"/>
       <c r="D6" s="28"/>
-      <c r="F6" s="365" t="s">
+      <c r="F6" s="404" t="s">
         <v>546</v>
       </c>
-      <c r="G6" s="365"/>
+      <c r="G6" s="404"/>
     </row>
     <row r="7" spans="1:7" ht="15.75" customHeight="1">
       <c r="A7" s="33"/>
@@ -13554,16 +13553,16 @@
       <c r="G196" s="33"/>
     </row>
     <row r="197" spans="1:8" ht="33.75" customHeight="1">
-      <c r="A197" s="368" t="s">
+      <c r="A197" s="386" t="s">
         <v>745</v>
       </c>
-      <c r="B197" s="368"/>
-      <c r="C197" s="368"/>
-      <c r="D197" s="368"/>
-      <c r="E197" s="368"/>
-      <c r="F197" s="368"/>
-      <c r="G197" s="368"/>
-      <c r="H197" s="368"/>
+      <c r="B197" s="386"/>
+      <c r="C197" s="386"/>
+      <c r="D197" s="386"/>
+      <c r="E197" s="386"/>
+      <c r="F197" s="386"/>
+      <c r="G197" s="386"/>
+      <c r="H197" s="386"/>
     </row>
     <row r="198" spans="1:8">
       <c r="B198" s="22"/>
@@ -13574,52 +13573,52 @@
       <c r="G198" s="82"/>
     </row>
     <row r="199" spans="1:8" ht="18.75" customHeight="1">
-      <c r="A199" s="364" t="s">
+      <c r="A199" s="405" t="s">
         <v>648</v>
       </c>
-      <c r="B199" s="364"/>
-      <c r="C199" s="364"/>
-      <c r="D199" s="364"/>
-      <c r="E199" s="364"/>
-      <c r="F199" s="364"/>
-      <c r="G199" s="364"/>
-      <c r="H199" s="364"/>
+      <c r="B199" s="405"/>
+      <c r="C199" s="405"/>
+      <c r="D199" s="405"/>
+      <c r="E199" s="405"/>
+      <c r="F199" s="405"/>
+      <c r="G199" s="405"/>
+      <c r="H199" s="405"/>
     </row>
     <row r="200" spans="1:8" ht="31.5" customHeight="1">
-      <c r="A200" s="364" t="s">
+      <c r="A200" s="405" t="s">
         <v>653</v>
       </c>
-      <c r="B200" s="364"/>
-      <c r="C200" s="364"/>
-      <c r="D200" s="364"/>
-      <c r="E200" s="364"/>
-      <c r="F200" s="364"/>
-      <c r="G200" s="364"/>
-      <c r="H200" s="364"/>
+      <c r="B200" s="405"/>
+      <c r="C200" s="405"/>
+      <c r="D200" s="405"/>
+      <c r="E200" s="405"/>
+      <c r="F200" s="405"/>
+      <c r="G200" s="405"/>
+      <c r="H200" s="405"/>
     </row>
     <row r="201" spans="1:8" ht="18.75" customHeight="1">
-      <c r="A201" s="364" t="s">
+      <c r="A201" s="405" t="s">
         <v>652</v>
       </c>
-      <c r="B201" s="364"/>
-      <c r="C201" s="364"/>
-      <c r="D201" s="364"/>
-      <c r="E201" s="364"/>
-      <c r="F201" s="364"/>
-      <c r="G201" s="364"/>
-      <c r="H201" s="364"/>
+      <c r="B201" s="405"/>
+      <c r="C201" s="405"/>
+      <c r="D201" s="405"/>
+      <c r="E201" s="405"/>
+      <c r="F201" s="405"/>
+      <c r="G201" s="405"/>
+      <c r="H201" s="405"/>
     </row>
     <row r="202" spans="1:8" ht="18.75" customHeight="1">
-      <c r="A202" s="367" t="s">
+      <c r="A202" s="399" t="s">
         <v>689</v>
       </c>
-      <c r="B202" s="367"/>
-      <c r="C202" s="367"/>
-      <c r="D202" s="367"/>
-      <c r="E202" s="367"/>
-      <c r="F202" s="367"/>
-      <c r="G202" s="367"/>
-      <c r="H202" s="367"/>
+      <c r="B202" s="399"/>
+      <c r="C202" s="399"/>
+      <c r="D202" s="399"/>
+      <c r="E202" s="399"/>
+      <c r="F202" s="399"/>
+      <c r="G202" s="399"/>
+      <c r="H202" s="399"/>
     </row>
     <row r="203" spans="1:8" ht="18.75" customHeight="1">
       <c r="A203" s="22" t="s">
@@ -13634,16 +13633,16 @@
       <c r="H203"/>
     </row>
     <row r="204" spans="1:8" ht="18.75" customHeight="1">
-      <c r="A204" s="364" t="s">
+      <c r="A204" s="405" t="s">
         <v>656</v>
       </c>
-      <c r="B204" s="364"/>
-      <c r="C204" s="364"/>
-      <c r="D204" s="364"/>
-      <c r="E204" s="364"/>
-      <c r="F204" s="364"/>
-      <c r="G204" s="364"/>
-      <c r="H204" s="364"/>
+      <c r="B204" s="405"/>
+      <c r="C204" s="405"/>
+      <c r="D204" s="405"/>
+      <c r="E204" s="405"/>
+      <c r="F204" s="405"/>
+      <c r="G204" s="405"/>
+      <c r="H204" s="405"/>
     </row>
     <row r="205" spans="1:8" ht="18.75" customHeight="1">
       <c r="A205" s="22" t="s">
@@ -13658,16 +13657,16 @@
       <c r="H205"/>
     </row>
     <row r="206" spans="1:8" ht="18.75" customHeight="1">
-      <c r="A206" s="364" t="s">
+      <c r="A206" s="405" t="s">
         <v>681</v>
       </c>
-      <c r="B206" s="364"/>
-      <c r="C206" s="364"/>
-      <c r="D206" s="364"/>
-      <c r="E206" s="364"/>
-      <c r="F206" s="364"/>
-      <c r="G206" s="364"/>
-      <c r="H206" s="364"/>
+      <c r="B206" s="405"/>
+      <c r="C206" s="405"/>
+      <c r="D206" s="405"/>
+      <c r="E206" s="405"/>
+      <c r="F206" s="405"/>
+      <c r="G206" s="405"/>
+      <c r="H206" s="405"/>
     </row>
     <row r="207" spans="1:8" ht="18.75" customHeight="1">
       <c r="A207" s="22" t="s">
@@ -13796,17 +13795,17 @@
     </row>
     <row r="5" spans="1:7" ht="15.75" customHeight="1">
       <c r="A5" s="33"/>
-      <c r="F5" s="365" t="s">
+      <c r="F5" s="404" t="s">
         <v>548</v>
       </c>
-      <c r="G5" s="365"/>
+      <c r="G5" s="404"/>
     </row>
     <row r="6" spans="1:7" ht="15.75" customHeight="1">
       <c r="A6" s="33"/>
-      <c r="F6" s="365" t="s">
+      <c r="F6" s="404" t="s">
         <v>549</v>
       </c>
-      <c r="G6" s="365"/>
+      <c r="G6" s="404"/>
     </row>
     <row r="7" spans="1:7">
       <c r="A7" s="33"/>
@@ -14718,12 +14717,12 @@
       <c r="B5" s="22"/>
       <c r="C5" s="22"/>
       <c r="D5" s="22"/>
-      <c r="E5" s="365" t="s">
+      <c r="E5" s="404" t="s">
         <v>78</v>
       </c>
-      <c r="F5" s="365"/>
-      <c r="G5" s="365"/>
-      <c r="H5" s="365"/>
+      <c r="F5" s="404"/>
+      <c r="G5" s="404"/>
+      <c r="H5" s="404"/>
     </row>
     <row r="6" spans="1:8">
       <c r="A6" s="22"/>
@@ -19822,73 +19821,73 @@
       <c r="C196" s="22"/>
     </row>
     <row r="197" spans="1:9" ht="32.25" customHeight="1">
-      <c r="A197" s="368" t="s">
+      <c r="A197" s="386" t="s">
         <v>745</v>
       </c>
-      <c r="B197" s="368"/>
-      <c r="C197" s="368"/>
-      <c r="D197" s="368"/>
-      <c r="E197" s="368"/>
-      <c r="F197" s="368"/>
-      <c r="G197" s="368"/>
-      <c r="H197" s="368"/>
-      <c r="I197" s="368"/>
+      <c r="B197" s="386"/>
+      <c r="C197" s="386"/>
+      <c r="D197" s="386"/>
+      <c r="E197" s="386"/>
+      <c r="F197" s="386"/>
+      <c r="G197" s="386"/>
+      <c r="H197" s="386"/>
+      <c r="I197" s="386"/>
     </row>
     <row r="198" spans="1:9" ht="18">
       <c r="A198" s="88"/>
       <c r="B198" s="89"/>
     </row>
     <row r="199" spans="1:9" ht="18.75" customHeight="1">
-      <c r="A199" s="364" t="s">
+      <c r="A199" s="405" t="s">
         <v>648</v>
       </c>
-      <c r="B199" s="364"/>
-      <c r="C199" s="364"/>
-      <c r="D199" s="364"/>
-      <c r="E199" s="364"/>
-      <c r="F199" s="364"/>
-      <c r="G199" s="364"/>
-      <c r="H199" s="364"/>
-      <c r="I199" s="364"/>
+      <c r="B199" s="405"/>
+      <c r="C199" s="405"/>
+      <c r="D199" s="405"/>
+      <c r="E199" s="405"/>
+      <c r="F199" s="405"/>
+      <c r="G199" s="405"/>
+      <c r="H199" s="405"/>
+      <c r="I199" s="405"/>
     </row>
     <row r="200" spans="1:9" ht="18.75" customHeight="1">
-      <c r="A200" s="364" t="s">
+      <c r="A200" s="405" t="s">
         <v>653</v>
       </c>
-      <c r="B200" s="364"/>
-      <c r="C200" s="364"/>
-      <c r="D200" s="364"/>
-      <c r="E200" s="364"/>
-      <c r="F200" s="364"/>
-      <c r="G200" s="364"/>
-      <c r="H200" s="364"/>
-      <c r="I200" s="364"/>
+      <c r="B200" s="405"/>
+      <c r="C200" s="405"/>
+      <c r="D200" s="405"/>
+      <c r="E200" s="405"/>
+      <c r="F200" s="405"/>
+      <c r="G200" s="405"/>
+      <c r="H200" s="405"/>
+      <c r="I200" s="405"/>
     </row>
     <row r="201" spans="1:9" ht="18.75" customHeight="1">
-      <c r="A201" s="364" t="s">
+      <c r="A201" s="405" t="s">
         <v>652</v>
       </c>
-      <c r="B201" s="364"/>
-      <c r="C201" s="364"/>
-      <c r="D201" s="364"/>
-      <c r="E201" s="364"/>
-      <c r="F201" s="364"/>
-      <c r="G201" s="364"/>
-      <c r="H201" s="364"/>
-      <c r="I201" s="364"/>
+      <c r="B201" s="405"/>
+      <c r="C201" s="405"/>
+      <c r="D201" s="405"/>
+      <c r="E201" s="405"/>
+      <c r="F201" s="405"/>
+      <c r="G201" s="405"/>
+      <c r="H201" s="405"/>
+      <c r="I201" s="405"/>
     </row>
     <row r="202" spans="1:9" ht="18.75" customHeight="1">
-      <c r="A202" s="367" t="s">
+      <c r="A202" s="399" t="s">
         <v>689</v>
       </c>
-      <c r="B202" s="367"/>
-      <c r="C202" s="367"/>
-      <c r="D202" s="367"/>
-      <c r="E202" s="367"/>
-      <c r="F202" s="367"/>
-      <c r="G202" s="367"/>
-      <c r="H202" s="367"/>
-      <c r="I202" s="367"/>
+      <c r="B202" s="399"/>
+      <c r="C202" s="399"/>
+      <c r="D202" s="399"/>
+      <c r="E202" s="399"/>
+      <c r="F202" s="399"/>
+      <c r="G202" s="399"/>
+      <c r="H202" s="399"/>
+      <c r="I202" s="399"/>
     </row>
     <row r="203" spans="1:9" ht="18.75" customHeight="1">
       <c r="A203" s="22" t="s">
@@ -19904,17 +19903,17 @@
       <c r="I203"/>
     </row>
     <row r="204" spans="1:9" ht="18.75" customHeight="1">
-      <c r="A204" s="364" t="s">
+      <c r="A204" s="405" t="s">
         <v>656</v>
       </c>
-      <c r="B204" s="364"/>
-      <c r="C204" s="364"/>
-      <c r="D204" s="364"/>
-      <c r="E204" s="364"/>
-      <c r="F204" s="364"/>
-      <c r="G204" s="364"/>
-      <c r="H204" s="364"/>
-      <c r="I204" s="364"/>
+      <c r="B204" s="405"/>
+      <c r="C204" s="405"/>
+      <c r="D204" s="405"/>
+      <c r="E204" s="405"/>
+      <c r="F204" s="405"/>
+      <c r="G204" s="405"/>
+      <c r="H204" s="405"/>
+      <c r="I204" s="405"/>
     </row>
     <row r="205" spans="1:9" ht="18.75" customHeight="1">
       <c r="A205" s="22" t="s">
@@ -19930,17 +19929,17 @@
       <c r="I205"/>
     </row>
     <row r="206" spans="1:9" ht="18.75" customHeight="1">
-      <c r="A206" s="364" t="s">
+      <c r="A206" s="405" t="s">
         <v>681</v>
       </c>
-      <c r="B206" s="364"/>
-      <c r="C206" s="364"/>
-      <c r="D206" s="364"/>
-      <c r="E206" s="364"/>
-      <c r="F206" s="364"/>
-      <c r="G206" s="364"/>
-      <c r="H206" s="364"/>
-      <c r="I206" s="364"/>
+      <c r="B206" s="405"/>
+      <c r="C206" s="405"/>
+      <c r="D206" s="405"/>
+      <c r="E206" s="405"/>
+      <c r="F206" s="405"/>
+      <c r="G206" s="405"/>
+      <c r="H206" s="405"/>
+      <c r="I206" s="405"/>
     </row>
     <row r="207" spans="1:9" ht="18.75" customHeight="1">
       <c r="A207" s="22" t="s">
@@ -24468,17 +24467,17 @@
       <c r="C195" s="22"/>
     </row>
     <row r="196" spans="1:9" ht="31.5" customHeight="1">
-      <c r="A196" s="368" t="s">
+      <c r="A196" s="386" t="s">
         <v>745</v>
       </c>
-      <c r="B196" s="368"/>
-      <c r="C196" s="368"/>
-      <c r="D196" s="368"/>
-      <c r="E196" s="368"/>
-      <c r="F196" s="368"/>
-      <c r="G196" s="368"/>
-      <c r="H196" s="368"/>
-      <c r="I196" s="368"/>
+      <c r="B196" s="386"/>
+      <c r="C196" s="386"/>
+      <c r="D196" s="386"/>
+      <c r="E196" s="386"/>
+      <c r="F196" s="386"/>
+      <c r="G196" s="386"/>
+      <c r="H196" s="386"/>
+      <c r="I196" s="386"/>
     </row>
     <row r="197" spans="1:9">
       <c r="B197" s="22"/>
@@ -24491,56 +24490,56 @@
       <c r="I197" s="91"/>
     </row>
     <row r="198" spans="1:9" ht="18.75" customHeight="1">
-      <c r="A198" s="364" t="s">
+      <c r="A198" s="405" t="s">
         <v>648</v>
       </c>
-      <c r="B198" s="364"/>
-      <c r="C198" s="364"/>
-      <c r="D198" s="364"/>
-      <c r="E198" s="364"/>
-      <c r="F198" s="364"/>
-      <c r="G198" s="364"/>
-      <c r="H198" s="364"/>
-      <c r="I198" s="364"/>
+      <c r="B198" s="405"/>
+      <c r="C198" s="405"/>
+      <c r="D198" s="405"/>
+      <c r="E198" s="405"/>
+      <c r="F198" s="405"/>
+      <c r="G198" s="405"/>
+      <c r="H198" s="405"/>
+      <c r="I198" s="405"/>
     </row>
     <row r="199" spans="1:9" ht="18.75" customHeight="1">
-      <c r="A199" s="364" t="s">
+      <c r="A199" s="405" t="s">
         <v>653</v>
       </c>
-      <c r="B199" s="364"/>
-      <c r="C199" s="364"/>
-      <c r="D199" s="364"/>
-      <c r="E199" s="364"/>
-      <c r="F199" s="364"/>
-      <c r="G199" s="364"/>
-      <c r="H199" s="364"/>
-      <c r="I199" s="364"/>
+      <c r="B199" s="405"/>
+      <c r="C199" s="405"/>
+      <c r="D199" s="405"/>
+      <c r="E199" s="405"/>
+      <c r="F199" s="405"/>
+      <c r="G199" s="405"/>
+      <c r="H199" s="405"/>
+      <c r="I199" s="405"/>
     </row>
     <row r="200" spans="1:9" ht="18.75" customHeight="1">
-      <c r="A200" s="364" t="s">
+      <c r="A200" s="405" t="s">
         <v>652</v>
       </c>
-      <c r="B200" s="364"/>
-      <c r="C200" s="364"/>
-      <c r="D200" s="364"/>
-      <c r="E200" s="364"/>
-      <c r="F200" s="364"/>
-      <c r="G200" s="364"/>
-      <c r="H200" s="364"/>
-      <c r="I200" s="364"/>
+      <c r="B200" s="405"/>
+      <c r="C200" s="405"/>
+      <c r="D200" s="405"/>
+      <c r="E200" s="405"/>
+      <c r="F200" s="405"/>
+      <c r="G200" s="405"/>
+      <c r="H200" s="405"/>
+      <c r="I200" s="405"/>
     </row>
     <row r="201" spans="1:9" ht="18.75" customHeight="1">
-      <c r="A201" s="367" t="s">
+      <c r="A201" s="399" t="s">
         <v>689</v>
       </c>
-      <c r="B201" s="367"/>
-      <c r="C201" s="367"/>
-      <c r="D201" s="367"/>
-      <c r="E201" s="367"/>
-      <c r="F201" s="367"/>
-      <c r="G201" s="367"/>
-      <c r="H201" s="367"/>
-      <c r="I201" s="367"/>
+      <c r="B201" s="399"/>
+      <c r="C201" s="399"/>
+      <c r="D201" s="399"/>
+      <c r="E201" s="399"/>
+      <c r="F201" s="399"/>
+      <c r="G201" s="399"/>
+      <c r="H201" s="399"/>
+      <c r="I201" s="399"/>
     </row>
     <row r="202" spans="1:9" ht="18.75" customHeight="1">
       <c r="A202" s="33" t="s">
@@ -24554,17 +24553,17 @@
       <c r="I202" s="33"/>
     </row>
     <row r="203" spans="1:9" ht="18.75" customHeight="1">
-      <c r="A203" s="364" t="s">
+      <c r="A203" s="405" t="s">
         <v>656</v>
       </c>
-      <c r="B203" s="364"/>
-      <c r="C203" s="364"/>
-      <c r="D203" s="364"/>
-      <c r="E203" s="364"/>
-      <c r="F203" s="364"/>
-      <c r="G203" s="364"/>
-      <c r="H203" s="364"/>
-      <c r="I203" s="364"/>
+      <c r="B203" s="405"/>
+      <c r="C203" s="405"/>
+      <c r="D203" s="405"/>
+      <c r="E203" s="405"/>
+      <c r="F203" s="405"/>
+      <c r="G203" s="405"/>
+      <c r="H203" s="405"/>
+      <c r="I203" s="405"/>
     </row>
     <row r="204" spans="1:9" ht="18.75" customHeight="1">
       <c r="A204" s="33" t="s">
@@ -24578,17 +24577,17 @@
       <c r="I204" s="33"/>
     </row>
     <row r="205" spans="1:9" ht="18.75" customHeight="1">
-      <c r="A205" s="364" t="s">
+      <c r="A205" s="405" t="s">
         <v>690</v>
       </c>
-      <c r="B205" s="364"/>
-      <c r="C205" s="364"/>
-      <c r="D205" s="364"/>
-      <c r="E205" s="364"/>
-      <c r="F205" s="364"/>
-      <c r="G205" s="364"/>
-      <c r="H205" s="364"/>
-      <c r="I205" s="364"/>
+      <c r="B205" s="405"/>
+      <c r="C205" s="405"/>
+      <c r="D205" s="405"/>
+      <c r="E205" s="405"/>
+      <c r="F205" s="405"/>
+      <c r="G205" s="405"/>
+      <c r="H205" s="405"/>
+      <c r="I205" s="405"/>
     </row>
     <row r="206" spans="1:9" ht="18.75" customHeight="1">
       <c r="A206" s="22" t="s">
@@ -24722,12 +24721,12 @@
       <c r="B5" s="22"/>
       <c r="C5" s="22"/>
       <c r="D5" s="22"/>
-      <c r="E5" s="365" t="s">
+      <c r="E5" s="404" t="s">
         <v>78</v>
       </c>
-      <c r="F5" s="365"/>
-      <c r="G5" s="365"/>
-      <c r="H5" s="365"/>
+      <c r="F5" s="404"/>
+      <c r="G5" s="404"/>
+      <c r="H5" s="404"/>
     </row>
     <row r="6" spans="1:8">
       <c r="B6" s="22"/>
@@ -25807,7 +25806,7 @@
       <c r="G5" s="93"/>
     </row>
     <row r="6" spans="1:9" ht="15.75" customHeight="1">
-      <c r="E6" s="365" t="s">
+      <c r="E6" s="404" t="s">
         <v>82</v>
       </c>
       <c r="F6" s="407"/>
@@ -26349,13 +26348,13 @@
       <c r="J4" s="64"/>
     </row>
     <row r="5" spans="1:10">
-      <c r="F5" s="365" t="s">
+      <c r="F5" s="404" t="s">
         <v>82</v>
       </c>
-      <c r="G5" s="366"/>
-      <c r="H5" s="366"/>
-      <c r="I5" s="366"/>
-      <c r="J5" s="366"/>
+      <c r="G5" s="409"/>
+      <c r="H5" s="409"/>
+      <c r="I5" s="409"/>
+      <c r="J5" s="409"/>
     </row>
     <row r="6" spans="1:10" ht="15" customHeight="1">
       <c r="F6" s="121"/>
@@ -26550,12 +26549,8 @@
         <v>681.92499999999995</v>
       </c>
       <c r="E19" s="110"/>
-      <c r="F19" s="191">
-        <v>95.601512780462812</v>
-      </c>
-      <c r="G19" s="192">
-        <v>88.751744155240118</v>
-      </c>
+      <c r="F19" s="191"/>
+      <c r="G19" s="192"/>
       <c r="H19" s="187">
         <v>94.107269861055102</v>
       </c>
@@ -26588,9 +26583,7 @@
         <v>29.984000000000002</v>
       </c>
       <c r="E21" s="110"/>
-      <c r="F21" s="191">
-        <v>97.885538954108853</v>
-      </c>
+      <c r="F21" s="191"/>
       <c r="G21" s="187">
         <v>93.613260405549624</v>
       </c>
@@ -26972,9 +26965,7 @@
         <v>84.903570261437906</v>
       </c>
       <c r="E36" s="110"/>
-      <c r="F36" s="191">
-        <v>96.732595861560554</v>
-      </c>
+      <c r="F36" s="191"/>
       <c r="G36" s="187">
         <v>91.479174230434623</v>
       </c>
@@ -27664,9 +27655,7 @@
         <v>66.307000000000002</v>
       </c>
       <c r="E62" s="110"/>
-      <c r="F62" s="191">
-        <v>97.151130348228691</v>
-      </c>
+      <c r="F62" s="191"/>
       <c r="G62" s="187">
         <v>92.222540606572451</v>
       </c>
@@ -28132,9 +28121,7 @@
         <v>55.011429738562086</v>
       </c>
       <c r="E80" s="110"/>
-      <c r="F80" s="191">
-        <v>97.161839362259684</v>
-      </c>
+      <c r="F80" s="191"/>
       <c r="G80" s="187">
         <v>92.262490311356871</v>
       </c>
@@ -28404,9 +28391,7 @@
         <v>70.251000000000005</v>
       </c>
       <c r="E91" s="110"/>
-      <c r="F91" s="191">
-        <v>96.81428022376906</v>
-      </c>
+      <c r="F91" s="191"/>
       <c r="G91" s="187">
         <v>90.841411510156433</v>
       </c>
@@ -28844,9 +28829,7 @@
         <v>76.224999999999994</v>
       </c>
       <c r="E108" s="110"/>
-      <c r="F108" s="191">
-        <v>95.984257133486395</v>
-      </c>
+      <c r="F108" s="191"/>
       <c r="G108" s="187">
         <v>91.292882912430301</v>
       </c>
@@ -29200,9 +29183,7 @@
         <v>126.116</v>
       </c>
       <c r="E122" s="110"/>
-      <c r="F122" s="191">
-        <v>92.544165688731013</v>
-      </c>
+      <c r="F122" s="191"/>
       <c r="G122" s="187">
         <v>79.290955721139454</v>
       </c>
@@ -30144,9 +30125,7 @@
         <v>112.13567475035663</v>
       </c>
       <c r="E157" s="110"/>
-      <c r="F157" s="191">
-        <v>94.186939176034826</v>
-      </c>
+      <c r="F157" s="191"/>
       <c r="G157" s="187">
         <v>87.39463611865736</v>
       </c>
@@ -30726,9 +30705,7 @@
         <v>60.99132524964336</v>
       </c>
       <c r="E179" s="110"/>
-      <c r="F179" s="191">
-        <v>96.908601323744762</v>
-      </c>
+      <c r="F179" s="191"/>
       <c r="G179" s="187">
         <v>91.710476635448671</v>
       </c>
@@ -31197,18 +31174,18 @@
       <c r="J197" s="212"/>
     </row>
     <row r="198" spans="1:15" ht="32.25" customHeight="1">
-      <c r="A198" s="368" t="s">
+      <c r="A198" s="386" t="s">
         <v>745</v>
       </c>
-      <c r="B198" s="368"/>
-      <c r="C198" s="368"/>
-      <c r="D198" s="368"/>
-      <c r="E198" s="368"/>
-      <c r="F198" s="368"/>
-      <c r="G198" s="368"/>
-      <c r="H198" s="368"/>
-      <c r="I198" s="368"/>
-      <c r="J198" s="368"/>
+      <c r="B198" s="386"/>
+      <c r="C198" s="386"/>
+      <c r="D198" s="386"/>
+      <c r="E198" s="386"/>
+      <c r="F198" s="386"/>
+      <c r="G198" s="386"/>
+      <c r="H198" s="386"/>
+      <c r="I198" s="386"/>
+      <c r="J198" s="386"/>
     </row>
     <row r="199" spans="1:15" ht="15.75">
       <c r="A199" s="22"/>
@@ -31235,61 +31212,61 @@
       <c r="O201" s="2"/>
     </row>
     <row r="202" spans="1:15" ht="18.75" customHeight="1">
-      <c r="A202" s="364" t="s">
+      <c r="A202" s="405" t="s">
         <v>648</v>
       </c>
-      <c r="B202" s="364"/>
-      <c r="C202" s="364"/>
-      <c r="D202" s="364"/>
-      <c r="E202" s="364"/>
-      <c r="F202" s="364"/>
-      <c r="G202" s="364"/>
-      <c r="H202" s="364"/>
-      <c r="I202" s="364"/>
-      <c r="J202" s="364"/>
+      <c r="B202" s="405"/>
+      <c r="C202" s="405"/>
+      <c r="D202" s="405"/>
+      <c r="E202" s="405"/>
+      <c r="F202" s="405"/>
+      <c r="G202" s="405"/>
+      <c r="H202" s="405"/>
+      <c r="I202" s="405"/>
+      <c r="J202" s="405"/>
       <c r="K202" s="299"/>
     </row>
     <row r="203" spans="1:15" ht="18.75" customHeight="1">
-      <c r="A203" s="364" t="s">
+      <c r="A203" s="405" t="s">
         <v>653</v>
       </c>
-      <c r="B203" s="364"/>
-      <c r="C203" s="364"/>
-      <c r="D203" s="364"/>
-      <c r="E203" s="364"/>
-      <c r="F203" s="364"/>
-      <c r="G203" s="364"/>
-      <c r="H203" s="364"/>
-      <c r="I203" s="364"/>
-      <c r="J203" s="364"/>
+      <c r="B203" s="405"/>
+      <c r="C203" s="405"/>
+      <c r="D203" s="405"/>
+      <c r="E203" s="405"/>
+      <c r="F203" s="405"/>
+      <c r="G203" s="405"/>
+      <c r="H203" s="405"/>
+      <c r="I203" s="405"/>
+      <c r="J203" s="405"/>
     </row>
     <row r="204" spans="1:15" ht="38.25" customHeight="1">
-      <c r="A204" s="364" t="s">
+      <c r="A204" s="405" t="s">
         <v>655</v>
       </c>
-      <c r="B204" s="364"/>
-      <c r="C204" s="364"/>
-      <c r="D204" s="364"/>
-      <c r="E204" s="364"/>
-      <c r="F204" s="364"/>
-      <c r="G204" s="364"/>
-      <c r="H204" s="364"/>
-      <c r="I204" s="364"/>
-      <c r="J204" s="364"/>
+      <c r="B204" s="405"/>
+      <c r="C204" s="405"/>
+      <c r="D204" s="405"/>
+      <c r="E204" s="405"/>
+      <c r="F204" s="405"/>
+      <c r="G204" s="405"/>
+      <c r="H204" s="405"/>
+      <c r="I204" s="405"/>
+      <c r="J204" s="405"/>
     </row>
     <row r="205" spans="1:15" ht="19.5" customHeight="1">
-      <c r="A205" s="367" t="s">
+      <c r="A205" s="399" t="s">
         <v>689</v>
       </c>
-      <c r="B205" s="367"/>
-      <c r="C205" s="367"/>
-      <c r="D205" s="367"/>
-      <c r="E205" s="367"/>
-      <c r="F205" s="367"/>
-      <c r="G205" s="367"/>
-      <c r="H205" s="367"/>
-      <c r="I205" s="367"/>
-      <c r="J205" s="367"/>
+      <c r="B205" s="399"/>
+      <c r="C205" s="399"/>
+      <c r="D205" s="399"/>
+      <c r="E205" s="399"/>
+      <c r="F205" s="399"/>
+      <c r="G205" s="399"/>
+      <c r="H205" s="399"/>
+      <c r="I205" s="399"/>
+      <c r="J205" s="399"/>
     </row>
     <row r="206" spans="1:15" ht="18.75">
       <c r="A206" s="22" t="s">
@@ -31302,33 +31279,33 @@
       <c r="J206" s="64"/>
     </row>
     <row r="207" spans="1:15" ht="34.5" customHeight="1">
-      <c r="A207" s="367" t="s">
+      <c r="A207" s="399" t="s">
         <v>691</v>
       </c>
-      <c r="B207" s="367"/>
-      <c r="C207" s="367"/>
-      <c r="D207" s="367"/>
-      <c r="E207" s="367"/>
-      <c r="F207" s="367"/>
-      <c r="G207" s="367"/>
-      <c r="H207" s="367"/>
-      <c r="I207" s="367"/>
-      <c r="J207" s="367"/>
+      <c r="B207" s="399"/>
+      <c r="C207" s="399"/>
+      <c r="D207" s="399"/>
+      <c r="E207" s="399"/>
+      <c r="F207" s="399"/>
+      <c r="G207" s="399"/>
+      <c r="H207" s="399"/>
+      <c r="I207" s="399"/>
+      <c r="J207" s="399"/>
       <c r="K207" s="299"/>
     </row>
     <row r="208" spans="1:15" ht="18.75" customHeight="1">
-      <c r="A208" s="364" t="s">
+      <c r="A208" s="405" t="s">
         <v>692</v>
       </c>
-      <c r="B208" s="364"/>
-      <c r="C208" s="364"/>
-      <c r="D208" s="364"/>
-      <c r="E208" s="364"/>
-      <c r="F208" s="364"/>
-      <c r="G208" s="364"/>
-      <c r="H208" s="364"/>
-      <c r="I208" s="364"/>
-      <c r="J208" s="364"/>
+      <c r="B208" s="405"/>
+      <c r="C208" s="405"/>
+      <c r="D208" s="405"/>
+      <c r="E208" s="405"/>
+      <c r="F208" s="405"/>
+      <c r="G208" s="405"/>
+      <c r="H208" s="405"/>
+      <c r="I208" s="405"/>
+      <c r="J208" s="405"/>
     </row>
     <row r="209" spans="1:10" ht="18.75">
       <c r="A209" s="22" t="s">
@@ -31341,46 +31318,46 @@
       <c r="J209" s="64"/>
     </row>
     <row r="210" spans="1:10" ht="34.5" customHeight="1">
-      <c r="A210" s="364" t="s">
+      <c r="A210" s="405" t="s">
         <v>740</v>
       </c>
-      <c r="B210" s="364"/>
-      <c r="C210" s="364"/>
-      <c r="D210" s="364"/>
-      <c r="E210" s="364"/>
-      <c r="F210" s="364"/>
-      <c r="G210" s="364"/>
-      <c r="H210" s="364"/>
-      <c r="I210" s="364"/>
-      <c r="J210" s="364"/>
+      <c r="B210" s="405"/>
+      <c r="C210" s="405"/>
+      <c r="D210" s="405"/>
+      <c r="E210" s="405"/>
+      <c r="F210" s="405"/>
+      <c r="G210" s="405"/>
+      <c r="H210" s="405"/>
+      <c r="I210" s="405"/>
+      <c r="J210" s="405"/>
     </row>
     <row r="211" spans="1:10" ht="18.75" customHeight="1">
-      <c r="A211" s="364" t="s">
+      <c r="A211" s="405" t="s">
         <v>694</v>
       </c>
-      <c r="B211" s="364"/>
-      <c r="C211" s="364"/>
-      <c r="D211" s="364"/>
-      <c r="E211" s="364"/>
-      <c r="F211" s="364"/>
-      <c r="G211" s="364"/>
-      <c r="H211" s="364"/>
-      <c r="I211" s="364"/>
-      <c r="J211" s="364"/>
+      <c r="B211" s="405"/>
+      <c r="C211" s="405"/>
+      <c r="D211" s="405"/>
+      <c r="E211" s="405"/>
+      <c r="F211" s="405"/>
+      <c r="G211" s="405"/>
+      <c r="H211" s="405"/>
+      <c r="I211" s="405"/>
+      <c r="J211" s="405"/>
     </row>
     <row r="212" spans="1:10" ht="18.75">
-      <c r="A212" s="363" t="s">
+      <c r="A212" s="408" t="s">
         <v>695</v>
       </c>
-      <c r="B212" s="363"/>
-      <c r="C212" s="363"/>
-      <c r="D212" s="363"/>
-      <c r="E212" s="363"/>
-      <c r="F212" s="363"/>
-      <c r="G212" s="363"/>
-      <c r="H212" s="363"/>
-      <c r="I212" s="363"/>
-      <c r="J212" s="363"/>
+      <c r="B212" s="408"/>
+      <c r="C212" s="408"/>
+      <c r="D212" s="408"/>
+      <c r="E212" s="408"/>
+      <c r="F212" s="408"/>
+      <c r="G212" s="408"/>
+      <c r="H212" s="408"/>
+      <c r="I212" s="408"/>
+      <c r="J212" s="408"/>
     </row>
     <row r="213" spans="1:10" ht="15.75">
       <c r="A213" s="22"/>
@@ -31530,7 +31507,7 @@
       <c r="J4" s="22"/>
     </row>
     <row r="5" spans="1:10" ht="15" customHeight="1">
-      <c r="F5" s="365" t="s">
+      <c r="F5" s="404" t="s">
         <v>87</v>
       </c>
       <c r="G5" s="407"/>
@@ -36181,18 +36158,18 @@
       <c r="J196" s="22"/>
     </row>
     <row r="197" spans="1:15" ht="30.75" customHeight="1">
-      <c r="A197" s="368" t="s">
+      <c r="A197" s="386" t="s">
         <v>745</v>
       </c>
-      <c r="B197" s="368"/>
-      <c r="C197" s="368"/>
-      <c r="D197" s="368"/>
-      <c r="E197" s="368"/>
-      <c r="F197" s="368"/>
-      <c r="G197" s="368"/>
-      <c r="H197" s="368"/>
-      <c r="I197" s="368"/>
-      <c r="J197" s="368"/>
+      <c r="B197" s="386"/>
+      <c r="C197" s="386"/>
+      <c r="D197" s="386"/>
+      <c r="E197" s="386"/>
+      <c r="F197" s="386"/>
+      <c r="G197" s="386"/>
+      <c r="H197" s="386"/>
+      <c r="I197" s="386"/>
+      <c r="J197" s="386"/>
       <c r="K197" s="297"/>
     </row>
     <row r="198" spans="1:15">
@@ -36216,150 +36193,150 @@
       <c r="O200" s="2"/>
     </row>
     <row r="201" spans="1:15" s="170" customFormat="1" ht="18.75" customHeight="1">
-      <c r="A201" s="368" t="s">
+      <c r="A201" s="386" t="s">
         <v>648</v>
       </c>
-      <c r="B201" s="368"/>
-      <c r="C201" s="368"/>
-      <c r="D201" s="368"/>
-      <c r="E201" s="368"/>
-      <c r="F201" s="368"/>
-      <c r="G201" s="368"/>
-      <c r="H201" s="368"/>
-      <c r="I201" s="368"/>
-      <c r="J201" s="368"/>
+      <c r="B201" s="386"/>
+      <c r="C201" s="386"/>
+      <c r="D201" s="386"/>
+      <c r="E201" s="386"/>
+      <c r="F201" s="386"/>
+      <c r="G201" s="386"/>
+      <c r="H201" s="386"/>
+      <c r="I201" s="386"/>
+      <c r="J201" s="386"/>
       <c r="K201" s="299"/>
     </row>
     <row r="202" spans="1:15" s="170" customFormat="1" ht="18.75" customHeight="1">
-      <c r="A202" s="368" t="s">
+      <c r="A202" s="386" t="s">
         <v>653</v>
       </c>
-      <c r="B202" s="368"/>
-      <c r="C202" s="368"/>
-      <c r="D202" s="368"/>
-      <c r="E202" s="368"/>
-      <c r="F202" s="368"/>
-      <c r="G202" s="368"/>
-      <c r="H202" s="368"/>
-      <c r="I202" s="368"/>
-      <c r="J202" s="368"/>
+      <c r="B202" s="386"/>
+      <c r="C202" s="386"/>
+      <c r="D202" s="386"/>
+      <c r="E202" s="386"/>
+      <c r="F202" s="386"/>
+      <c r="G202" s="386"/>
+      <c r="H202" s="386"/>
+      <c r="I202" s="386"/>
+      <c r="J202" s="386"/>
       <c r="K202" s="299"/>
     </row>
     <row r="203" spans="1:15" s="170" customFormat="1" ht="33" customHeight="1">
-      <c r="A203" s="368" t="s">
+      <c r="A203" s="386" t="s">
         <v>655</v>
       </c>
-      <c r="B203" s="368"/>
-      <c r="C203" s="368"/>
-      <c r="D203" s="368"/>
-      <c r="E203" s="368"/>
-      <c r="F203" s="368"/>
-      <c r="G203" s="368"/>
-      <c r="H203" s="368"/>
-      <c r="I203" s="368"/>
-      <c r="J203" s="368"/>
+      <c r="B203" s="386"/>
+      <c r="C203" s="386"/>
+      <c r="D203" s="386"/>
+      <c r="E203" s="386"/>
+      <c r="F203" s="386"/>
+      <c r="G203" s="386"/>
+      <c r="H203" s="386"/>
+      <c r="I203" s="386"/>
+      <c r="J203" s="386"/>
       <c r="K203" s="299"/>
     </row>
     <row r="204" spans="1:15" s="170" customFormat="1" ht="18.75" customHeight="1">
-      <c r="A204" s="368" t="s">
+      <c r="A204" s="386" t="s">
         <v>689</v>
       </c>
-      <c r="B204" s="368"/>
-      <c r="C204" s="368"/>
-      <c r="D204" s="368"/>
-      <c r="E204" s="368"/>
-      <c r="F204" s="368"/>
-      <c r="G204" s="368"/>
-      <c r="H204" s="368"/>
-      <c r="I204" s="368"/>
-      <c r="J204" s="368"/>
+      <c r="B204" s="386"/>
+      <c r="C204" s="386"/>
+      <c r="D204" s="386"/>
+      <c r="E204" s="386"/>
+      <c r="F204" s="386"/>
+      <c r="G204" s="386"/>
+      <c r="H204" s="386"/>
+      <c r="I204" s="386"/>
+      <c r="J204" s="386"/>
       <c r="K204" s="299"/>
     </row>
     <row r="205" spans="1:15" s="299" customFormat="1" ht="18.75" customHeight="1">
-      <c r="A205" s="368" t="s">
+      <c r="A205" s="386" t="s">
         <v>748</v>
       </c>
-      <c r="B205" s="368"/>
-      <c r="C205" s="368"/>
-      <c r="D205" s="368"/>
-      <c r="E205" s="368"/>
-      <c r="F205" s="368"/>
-      <c r="G205" s="368"/>
-      <c r="H205" s="368"/>
-      <c r="I205" s="368"/>
-      <c r="J205" s="368"/>
+      <c r="B205" s="386"/>
+      <c r="C205" s="386"/>
+      <c r="D205" s="386"/>
+      <c r="E205" s="386"/>
+      <c r="F205" s="386"/>
+      <c r="G205" s="386"/>
+      <c r="H205" s="386"/>
+      <c r="I205" s="386"/>
+      <c r="J205" s="386"/>
       <c r="K205" s="44"/>
     </row>
     <row r="206" spans="1:15" s="299" customFormat="1" ht="34.5" customHeight="1">
-      <c r="A206" s="368" t="s">
+      <c r="A206" s="386" t="s">
         <v>691</v>
       </c>
-      <c r="B206" s="368"/>
-      <c r="C206" s="368"/>
-      <c r="D206" s="368"/>
-      <c r="E206" s="368"/>
-      <c r="F206" s="368"/>
-      <c r="G206" s="368"/>
-      <c r="H206" s="368"/>
-      <c r="I206" s="368"/>
-      <c r="J206" s="368"/>
+      <c r="B206" s="386"/>
+      <c r="C206" s="386"/>
+      <c r="D206" s="386"/>
+      <c r="E206" s="386"/>
+      <c r="F206" s="386"/>
+      <c r="G206" s="386"/>
+      <c r="H206" s="386"/>
+      <c r="I206" s="386"/>
+      <c r="J206" s="386"/>
     </row>
     <row r="207" spans="1:15" s="299" customFormat="1" ht="18.75" customHeight="1">
-      <c r="A207" s="368" t="s">
+      <c r="A207" s="386" t="s">
         <v>692</v>
       </c>
-      <c r="B207" s="368"/>
-      <c r="C207" s="368"/>
-      <c r="D207" s="368"/>
-      <c r="E207" s="368"/>
-      <c r="F207" s="368"/>
-      <c r="G207" s="368"/>
-      <c r="H207" s="368"/>
-      <c r="I207" s="368"/>
-      <c r="J207" s="368"/>
+      <c r="B207" s="386"/>
+      <c r="C207" s="386"/>
+      <c r="D207" s="386"/>
+      <c r="E207" s="386"/>
+      <c r="F207" s="386"/>
+      <c r="G207" s="386"/>
+      <c r="H207" s="386"/>
+      <c r="I207" s="386"/>
+      <c r="J207" s="386"/>
     </row>
     <row r="208" spans="1:15" s="299" customFormat="1" ht="18.75" customHeight="1">
-      <c r="A208" s="368" t="s">
+      <c r="A208" s="386" t="s">
         <v>693</v>
       </c>
-      <c r="B208" s="368"/>
-      <c r="C208" s="368"/>
-      <c r="D208" s="368"/>
-      <c r="E208" s="368"/>
-      <c r="F208" s="368"/>
-      <c r="G208" s="368"/>
-      <c r="H208" s="368"/>
-      <c r="I208" s="368"/>
-      <c r="J208" s="368"/>
+      <c r="B208" s="386"/>
+      <c r="C208" s="386"/>
+      <c r="D208" s="386"/>
+      <c r="E208" s="386"/>
+      <c r="F208" s="386"/>
+      <c r="G208" s="386"/>
+      <c r="H208" s="386"/>
+      <c r="I208" s="386"/>
+      <c r="J208" s="386"/>
       <c r="K208" s="44"/>
     </row>
     <row r="209" spans="1:11" s="299" customFormat="1" ht="34.5" customHeight="1">
-      <c r="A209" s="368" t="s">
+      <c r="A209" s="386" t="s">
         <v>741</v>
       </c>
-      <c r="B209" s="368"/>
-      <c r="C209" s="368"/>
-      <c r="D209" s="368"/>
-      <c r="E209" s="368"/>
-      <c r="F209" s="368"/>
-      <c r="G209" s="368"/>
-      <c r="H209" s="368"/>
-      <c r="I209" s="368"/>
-      <c r="J209" s="368"/>
+      <c r="B209" s="386"/>
+      <c r="C209" s="386"/>
+      <c r="D209" s="386"/>
+      <c r="E209" s="386"/>
+      <c r="F209" s="386"/>
+      <c r="G209" s="386"/>
+      <c r="H209" s="386"/>
+      <c r="I209" s="386"/>
+      <c r="J209" s="386"/>
     </row>
     <row r="210" spans="1:11" s="299" customFormat="1" ht="18.75" customHeight="1">
-      <c r="A210" s="368" t="s">
+      <c r="A210" s="386" t="s">
         <v>694</v>
       </c>
-      <c r="B210" s="368"/>
-      <c r="C210" s="368"/>
-      <c r="D210" s="368"/>
-      <c r="E210" s="368"/>
-      <c r="F210" s="368"/>
-      <c r="G210" s="368"/>
-      <c r="H210" s="368"/>
-      <c r="I210" s="368"/>
-      <c r="J210" s="368"/>
+      <c r="B210" s="386"/>
+      <c r="C210" s="386"/>
+      <c r="D210" s="386"/>
+      <c r="E210" s="386"/>
+      <c r="F210" s="386"/>
+      <c r="G210" s="386"/>
+      <c r="H210" s="386"/>
+      <c r="I210" s="386"/>
+      <c r="J210" s="386"/>
     </row>
     <row r="211" spans="1:11" s="299" customFormat="1" ht="18.75" customHeight="1">
       <c r="A211" s="44" t="s">
@@ -36457,11 +36434,6 @@
     <sortCondition ref="B180:B194"/>
   </sortState>
   <mergeCells count="12">
-    <mergeCell ref="F5:J5"/>
-    <mergeCell ref="A197:J197"/>
-    <mergeCell ref="A201:J201"/>
-    <mergeCell ref="A202:J202"/>
-    <mergeCell ref="A208:J208"/>
     <mergeCell ref="A209:J209"/>
     <mergeCell ref="A210:J210"/>
     <mergeCell ref="A203:J203"/>
@@ -36469,6 +36441,11 @@
     <mergeCell ref="A205:J205"/>
     <mergeCell ref="A206:J206"/>
     <mergeCell ref="A207:J207"/>
+    <mergeCell ref="F5:J5"/>
+    <mergeCell ref="A197:J197"/>
+    <mergeCell ref="A201:J201"/>
+    <mergeCell ref="A202:J202"/>
+    <mergeCell ref="A208:J208"/>
   </mergeCells>
   <pageMargins left="0.51181102362204722" right="0.51181102362204722" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" scale="54" fitToHeight="0" orientation="portrait" r:id="rId1"/>
@@ -36484,446 +36461,446 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="2" spans="1:9">
-      <c r="A2" s="369" t="s">
+      <c r="A2" s="365" t="s">
         <v>735</v>
       </c>
-      <c r="B2" s="370"/>
-      <c r="C2" s="370"/>
-      <c r="D2" s="370"/>
-      <c r="E2" s="370"/>
-      <c r="F2" s="370"/>
-      <c r="G2" s="370"/>
-      <c r="H2" s="370"/>
-      <c r="I2" s="371"/>
+      <c r="B2" s="366"/>
+      <c r="C2" s="366"/>
+      <c r="D2" s="366"/>
+      <c r="E2" s="366"/>
+      <c r="F2" s="366"/>
+      <c r="G2" s="366"/>
+      <c r="H2" s="366"/>
+      <c r="I2" s="367"/>
     </row>
     <row r="3" spans="1:9">
-      <c r="A3" s="372"/>
-      <c r="B3" s="373"/>
-      <c r="C3" s="373"/>
-      <c r="D3" s="373"/>
-      <c r="E3" s="373"/>
-      <c r="F3" s="373"/>
-      <c r="G3" s="373"/>
-      <c r="H3" s="373"/>
-      <c r="I3" s="374"/>
+      <c r="A3" s="368"/>
+      <c r="B3" s="369"/>
+      <c r="C3" s="369"/>
+      <c r="D3" s="369"/>
+      <c r="E3" s="369"/>
+      <c r="F3" s="369"/>
+      <c r="G3" s="369"/>
+      <c r="H3" s="369"/>
+      <c r="I3" s="370"/>
     </row>
     <row r="4" spans="1:9">
-      <c r="A4" s="372"/>
-      <c r="B4" s="373"/>
-      <c r="C4" s="373"/>
-      <c r="D4" s="373"/>
-      <c r="E4" s="373"/>
-      <c r="F4" s="373"/>
-      <c r="G4" s="373"/>
-      <c r="H4" s="373"/>
-      <c r="I4" s="374"/>
+      <c r="A4" s="368"/>
+      <c r="B4" s="369"/>
+      <c r="C4" s="369"/>
+      <c r="D4" s="369"/>
+      <c r="E4" s="369"/>
+      <c r="F4" s="369"/>
+      <c r="G4" s="369"/>
+      <c r="H4" s="369"/>
+      <c r="I4" s="370"/>
     </row>
     <row r="5" spans="1:9">
-      <c r="A5" s="372"/>
-      <c r="B5" s="373"/>
-      <c r="C5" s="373"/>
-      <c r="D5" s="373"/>
-      <c r="E5" s="373"/>
-      <c r="F5" s="373"/>
-      <c r="G5" s="373"/>
-      <c r="H5" s="373"/>
-      <c r="I5" s="374"/>
+      <c r="A5" s="368"/>
+      <c r="B5" s="369"/>
+      <c r="C5" s="369"/>
+      <c r="D5" s="369"/>
+      <c r="E5" s="369"/>
+      <c r="F5" s="369"/>
+      <c r="G5" s="369"/>
+      <c r="H5" s="369"/>
+      <c r="I5" s="370"/>
     </row>
     <row r="6" spans="1:9">
-      <c r="A6" s="372"/>
-      <c r="B6" s="373"/>
-      <c r="C6" s="373"/>
-      <c r="D6" s="373"/>
-      <c r="E6" s="373"/>
-      <c r="F6" s="373"/>
-      <c r="G6" s="373"/>
-      <c r="H6" s="373"/>
-      <c r="I6" s="374"/>
+      <c r="A6" s="368"/>
+      <c r="B6" s="369"/>
+      <c r="C6" s="369"/>
+      <c r="D6" s="369"/>
+      <c r="E6" s="369"/>
+      <c r="F6" s="369"/>
+      <c r="G6" s="369"/>
+      <c r="H6" s="369"/>
+      <c r="I6" s="370"/>
     </row>
     <row r="7" spans="1:9">
-      <c r="A7" s="372"/>
-      <c r="B7" s="373"/>
-      <c r="C7" s="373"/>
-      <c r="D7" s="373"/>
-      <c r="E7" s="373"/>
-      <c r="F7" s="373"/>
-      <c r="G7" s="373"/>
-      <c r="H7" s="373"/>
-      <c r="I7" s="374"/>
+      <c r="A7" s="368"/>
+      <c r="B7" s="369"/>
+      <c r="C7" s="369"/>
+      <c r="D7" s="369"/>
+      <c r="E7" s="369"/>
+      <c r="F7" s="369"/>
+      <c r="G7" s="369"/>
+      <c r="H7" s="369"/>
+      <c r="I7" s="370"/>
     </row>
     <row r="8" spans="1:9">
-      <c r="A8" s="372"/>
-      <c r="B8" s="373"/>
-      <c r="C8" s="373"/>
-      <c r="D8" s="373"/>
-      <c r="E8" s="373"/>
-      <c r="F8" s="373"/>
-      <c r="G8" s="373"/>
-      <c r="H8" s="373"/>
-      <c r="I8" s="374"/>
+      <c r="A8" s="368"/>
+      <c r="B8" s="369"/>
+      <c r="C8" s="369"/>
+      <c r="D8" s="369"/>
+      <c r="E8" s="369"/>
+      <c r="F8" s="369"/>
+      <c r="G8" s="369"/>
+      <c r="H8" s="369"/>
+      <c r="I8" s="370"/>
     </row>
     <row r="9" spans="1:9">
-      <c r="A9" s="372"/>
-      <c r="B9" s="373"/>
-      <c r="C9" s="373"/>
-      <c r="D9" s="373"/>
-      <c r="E9" s="373"/>
-      <c r="F9" s="373"/>
-      <c r="G9" s="373"/>
-      <c r="H9" s="373"/>
-      <c r="I9" s="374"/>
+      <c r="A9" s="368"/>
+      <c r="B9" s="369"/>
+      <c r="C9" s="369"/>
+      <c r="D9" s="369"/>
+      <c r="E9" s="369"/>
+      <c r="F9" s="369"/>
+      <c r="G9" s="369"/>
+      <c r="H9" s="369"/>
+      <c r="I9" s="370"/>
     </row>
     <row r="10" spans="1:9">
-      <c r="A10" s="372"/>
-      <c r="B10" s="373"/>
-      <c r="C10" s="373"/>
-      <c r="D10" s="373"/>
-      <c r="E10" s="373"/>
-      <c r="F10" s="373"/>
-      <c r="G10" s="373"/>
-      <c r="H10" s="373"/>
-      <c r="I10" s="374"/>
+      <c r="A10" s="368"/>
+      <c r="B10" s="369"/>
+      <c r="C10" s="369"/>
+      <c r="D10" s="369"/>
+      <c r="E10" s="369"/>
+      <c r="F10" s="369"/>
+      <c r="G10" s="369"/>
+      <c r="H10" s="369"/>
+      <c r="I10" s="370"/>
     </row>
     <row r="11" spans="1:9">
-      <c r="A11" s="372"/>
-      <c r="B11" s="373"/>
-      <c r="C11" s="373"/>
-      <c r="D11" s="373"/>
-      <c r="E11" s="373"/>
-      <c r="F11" s="373"/>
-      <c r="G11" s="373"/>
-      <c r="H11" s="373"/>
-      <c r="I11" s="374"/>
+      <c r="A11" s="368"/>
+      <c r="B11" s="369"/>
+      <c r="C11" s="369"/>
+      <c r="D11" s="369"/>
+      <c r="E11" s="369"/>
+      <c r="F11" s="369"/>
+      <c r="G11" s="369"/>
+      <c r="H11" s="369"/>
+      <c r="I11" s="370"/>
     </row>
     <row r="12" spans="1:9">
-      <c r="A12" s="372"/>
-      <c r="B12" s="373"/>
-      <c r="C12" s="373"/>
-      <c r="D12" s="373"/>
-      <c r="E12" s="373"/>
-      <c r="F12" s="373"/>
-      <c r="G12" s="373"/>
-      <c r="H12" s="373"/>
-      <c r="I12" s="374"/>
+      <c r="A12" s="368"/>
+      <c r="B12" s="369"/>
+      <c r="C12" s="369"/>
+      <c r="D12" s="369"/>
+      <c r="E12" s="369"/>
+      <c r="F12" s="369"/>
+      <c r="G12" s="369"/>
+      <c r="H12" s="369"/>
+      <c r="I12" s="370"/>
     </row>
     <row r="13" spans="1:9">
-      <c r="A13" s="372"/>
-      <c r="B13" s="373"/>
-      <c r="C13" s="373"/>
-      <c r="D13" s="373"/>
-      <c r="E13" s="373"/>
-      <c r="F13" s="373"/>
-      <c r="G13" s="373"/>
-      <c r="H13" s="373"/>
-      <c r="I13" s="374"/>
+      <c r="A13" s="368"/>
+      <c r="B13" s="369"/>
+      <c r="C13" s="369"/>
+      <c r="D13" s="369"/>
+      <c r="E13" s="369"/>
+      <c r="F13" s="369"/>
+      <c r="G13" s="369"/>
+      <c r="H13" s="369"/>
+      <c r="I13" s="370"/>
     </row>
     <row r="14" spans="1:9">
-      <c r="A14" s="372"/>
-      <c r="B14" s="373"/>
-      <c r="C14" s="373"/>
-      <c r="D14" s="373"/>
-      <c r="E14" s="373"/>
-      <c r="F14" s="373"/>
-      <c r="G14" s="373"/>
-      <c r="H14" s="373"/>
-      <c r="I14" s="374"/>
+      <c r="A14" s="368"/>
+      <c r="B14" s="369"/>
+      <c r="C14" s="369"/>
+      <c r="D14" s="369"/>
+      <c r="E14" s="369"/>
+      <c r="F14" s="369"/>
+      <c r="G14" s="369"/>
+      <c r="H14" s="369"/>
+      <c r="I14" s="370"/>
     </row>
     <row r="15" spans="1:9">
-      <c r="A15" s="372"/>
-      <c r="B15" s="373"/>
-      <c r="C15" s="373"/>
-      <c r="D15" s="373"/>
-      <c r="E15" s="373"/>
-      <c r="F15" s="373"/>
-      <c r="G15" s="373"/>
-      <c r="H15" s="373"/>
-      <c r="I15" s="374"/>
+      <c r="A15" s="368"/>
+      <c r="B15" s="369"/>
+      <c r="C15" s="369"/>
+      <c r="D15" s="369"/>
+      <c r="E15" s="369"/>
+      <c r="F15" s="369"/>
+      <c r="G15" s="369"/>
+      <c r="H15" s="369"/>
+      <c r="I15" s="370"/>
     </row>
     <row r="16" spans="1:9">
-      <c r="A16" s="372"/>
-      <c r="B16" s="373"/>
-      <c r="C16" s="373"/>
-      <c r="D16" s="373"/>
-      <c r="E16" s="373"/>
-      <c r="F16" s="373"/>
-      <c r="G16" s="373"/>
-      <c r="H16" s="373"/>
-      <c r="I16" s="374"/>
+      <c r="A16" s="368"/>
+      <c r="B16" s="369"/>
+      <c r="C16" s="369"/>
+      <c r="D16" s="369"/>
+      <c r="E16" s="369"/>
+      <c r="F16" s="369"/>
+      <c r="G16" s="369"/>
+      <c r="H16" s="369"/>
+      <c r="I16" s="370"/>
     </row>
     <row r="17" spans="1:9">
-      <c r="A17" s="372"/>
-      <c r="B17" s="373"/>
-      <c r="C17" s="373"/>
-      <c r="D17" s="373"/>
-      <c r="E17" s="373"/>
-      <c r="F17" s="373"/>
-      <c r="G17" s="373"/>
-      <c r="H17" s="373"/>
-      <c r="I17" s="374"/>
+      <c r="A17" s="368"/>
+      <c r="B17" s="369"/>
+      <c r="C17" s="369"/>
+      <c r="D17" s="369"/>
+      <c r="E17" s="369"/>
+      <c r="F17" s="369"/>
+      <c r="G17" s="369"/>
+      <c r="H17" s="369"/>
+      <c r="I17" s="370"/>
     </row>
     <row r="18" spans="1:9">
-      <c r="A18" s="372"/>
-      <c r="B18" s="373"/>
-      <c r="C18" s="373"/>
-      <c r="D18" s="373"/>
-      <c r="E18" s="373"/>
-      <c r="F18" s="373"/>
-      <c r="G18" s="373"/>
-      <c r="H18" s="373"/>
-      <c r="I18" s="374"/>
+      <c r="A18" s="368"/>
+      <c r="B18" s="369"/>
+      <c r="C18" s="369"/>
+      <c r="D18" s="369"/>
+      <c r="E18" s="369"/>
+      <c r="F18" s="369"/>
+      <c r="G18" s="369"/>
+      <c r="H18" s="369"/>
+      <c r="I18" s="370"/>
     </row>
     <row r="19" spans="1:9">
-      <c r="A19" s="372"/>
-      <c r="B19" s="373"/>
-      <c r="C19" s="373"/>
-      <c r="D19" s="373"/>
-      <c r="E19" s="373"/>
-      <c r="F19" s="373"/>
-      <c r="G19" s="373"/>
-      <c r="H19" s="373"/>
-      <c r="I19" s="374"/>
+      <c r="A19" s="368"/>
+      <c r="B19" s="369"/>
+      <c r="C19" s="369"/>
+      <c r="D19" s="369"/>
+      <c r="E19" s="369"/>
+      <c r="F19" s="369"/>
+      <c r="G19" s="369"/>
+      <c r="H19" s="369"/>
+      <c r="I19" s="370"/>
     </row>
     <row r="20" spans="1:9">
-      <c r="A20" s="372"/>
-      <c r="B20" s="373"/>
-      <c r="C20" s="373"/>
-      <c r="D20" s="373"/>
-      <c r="E20" s="373"/>
-      <c r="F20" s="373"/>
-      <c r="G20" s="373"/>
-      <c r="H20" s="373"/>
-      <c r="I20" s="374"/>
+      <c r="A20" s="368"/>
+      <c r="B20" s="369"/>
+      <c r="C20" s="369"/>
+      <c r="D20" s="369"/>
+      <c r="E20" s="369"/>
+      <c r="F20" s="369"/>
+      <c r="G20" s="369"/>
+      <c r="H20" s="369"/>
+      <c r="I20" s="370"/>
     </row>
     <row r="21" spans="1:9">
-      <c r="A21" s="372"/>
-      <c r="B21" s="373"/>
-      <c r="C21" s="373"/>
-      <c r="D21" s="373"/>
-      <c r="E21" s="373"/>
-      <c r="F21" s="373"/>
-      <c r="G21" s="373"/>
-      <c r="H21" s="373"/>
-      <c r="I21" s="374"/>
+      <c r="A21" s="368"/>
+      <c r="B21" s="369"/>
+      <c r="C21" s="369"/>
+      <c r="D21" s="369"/>
+      <c r="E21" s="369"/>
+      <c r="F21" s="369"/>
+      <c r="G21" s="369"/>
+      <c r="H21" s="369"/>
+      <c r="I21" s="370"/>
     </row>
     <row r="22" spans="1:9">
-      <c r="A22" s="372"/>
-      <c r="B22" s="373"/>
-      <c r="C22" s="373"/>
-      <c r="D22" s="373"/>
-      <c r="E22" s="373"/>
-      <c r="F22" s="373"/>
-      <c r="G22" s="373"/>
-      <c r="H22" s="373"/>
-      <c r="I22" s="374"/>
+      <c r="A22" s="368"/>
+      <c r="B22" s="369"/>
+      <c r="C22" s="369"/>
+      <c r="D22" s="369"/>
+      <c r="E22" s="369"/>
+      <c r="F22" s="369"/>
+      <c r="G22" s="369"/>
+      <c r="H22" s="369"/>
+      <c r="I22" s="370"/>
     </row>
     <row r="23" spans="1:9">
-      <c r="A23" s="372"/>
-      <c r="B23" s="373"/>
-      <c r="C23" s="373"/>
-      <c r="D23" s="373"/>
-      <c r="E23" s="373"/>
-      <c r="F23" s="373"/>
-      <c r="G23" s="373"/>
-      <c r="H23" s="373"/>
-      <c r="I23" s="374"/>
+      <c r="A23" s="368"/>
+      <c r="B23" s="369"/>
+      <c r="C23" s="369"/>
+      <c r="D23" s="369"/>
+      <c r="E23" s="369"/>
+      <c r="F23" s="369"/>
+      <c r="G23" s="369"/>
+      <c r="H23" s="369"/>
+      <c r="I23" s="370"/>
     </row>
     <row r="24" spans="1:9">
-      <c r="A24" s="372"/>
-      <c r="B24" s="373"/>
-      <c r="C24" s="373"/>
-      <c r="D24" s="373"/>
-      <c r="E24" s="373"/>
-      <c r="F24" s="373"/>
-      <c r="G24" s="373"/>
-      <c r="H24" s="373"/>
-      <c r="I24" s="374"/>
+      <c r="A24" s="368"/>
+      <c r="B24" s="369"/>
+      <c r="C24" s="369"/>
+      <c r="D24" s="369"/>
+      <c r="E24" s="369"/>
+      <c r="F24" s="369"/>
+      <c r="G24" s="369"/>
+      <c r="H24" s="369"/>
+      <c r="I24" s="370"/>
     </row>
     <row r="25" spans="1:9">
-      <c r="A25" s="372"/>
-      <c r="B25" s="373"/>
-      <c r="C25" s="373"/>
-      <c r="D25" s="373"/>
-      <c r="E25" s="373"/>
-      <c r="F25" s="373"/>
-      <c r="G25" s="373"/>
-      <c r="H25" s="373"/>
-      <c r="I25" s="374"/>
+      <c r="A25" s="368"/>
+      <c r="B25" s="369"/>
+      <c r="C25" s="369"/>
+      <c r="D25" s="369"/>
+      <c r="E25" s="369"/>
+      <c r="F25" s="369"/>
+      <c r="G25" s="369"/>
+      <c r="H25" s="369"/>
+      <c r="I25" s="370"/>
     </row>
     <row r="26" spans="1:9">
-      <c r="A26" s="372"/>
-      <c r="B26" s="373"/>
-      <c r="C26" s="373"/>
-      <c r="D26" s="373"/>
-      <c r="E26" s="373"/>
-      <c r="F26" s="373"/>
-      <c r="G26" s="373"/>
-      <c r="H26" s="373"/>
-      <c r="I26" s="374"/>
+      <c r="A26" s="368"/>
+      <c r="B26" s="369"/>
+      <c r="C26" s="369"/>
+      <c r="D26" s="369"/>
+      <c r="E26" s="369"/>
+      <c r="F26" s="369"/>
+      <c r="G26" s="369"/>
+      <c r="H26" s="369"/>
+      <c r="I26" s="370"/>
     </row>
     <row r="27" spans="1:9">
-      <c r="A27" s="372"/>
-      <c r="B27" s="373"/>
-      <c r="C27" s="373"/>
-      <c r="D27" s="373"/>
-      <c r="E27" s="373"/>
-      <c r="F27" s="373"/>
-      <c r="G27" s="373"/>
-      <c r="H27" s="373"/>
-      <c r="I27" s="374"/>
+      <c r="A27" s="368"/>
+      <c r="B27" s="369"/>
+      <c r="C27" s="369"/>
+      <c r="D27" s="369"/>
+      <c r="E27" s="369"/>
+      <c r="F27" s="369"/>
+      <c r="G27" s="369"/>
+      <c r="H27" s="369"/>
+      <c r="I27" s="370"/>
     </row>
     <row r="28" spans="1:9">
-      <c r="A28" s="372"/>
-      <c r="B28" s="373"/>
-      <c r="C28" s="373"/>
-      <c r="D28" s="373"/>
-      <c r="E28" s="373"/>
-      <c r="F28" s="373"/>
-      <c r="G28" s="373"/>
-      <c r="H28" s="373"/>
-      <c r="I28" s="374"/>
+      <c r="A28" s="368"/>
+      <c r="B28" s="369"/>
+      <c r="C28" s="369"/>
+      <c r="D28" s="369"/>
+      <c r="E28" s="369"/>
+      <c r="F28" s="369"/>
+      <c r="G28" s="369"/>
+      <c r="H28" s="369"/>
+      <c r="I28" s="370"/>
     </row>
     <row r="29" spans="1:9">
-      <c r="A29" s="372"/>
-      <c r="B29" s="373"/>
-      <c r="C29" s="373"/>
-      <c r="D29" s="373"/>
-      <c r="E29" s="373"/>
-      <c r="F29" s="373"/>
-      <c r="G29" s="373"/>
-      <c r="H29" s="373"/>
-      <c r="I29" s="374"/>
+      <c r="A29" s="368"/>
+      <c r="B29" s="369"/>
+      <c r="C29" s="369"/>
+      <c r="D29" s="369"/>
+      <c r="E29" s="369"/>
+      <c r="F29" s="369"/>
+      <c r="G29" s="369"/>
+      <c r="H29" s="369"/>
+      <c r="I29" s="370"/>
     </row>
     <row r="30" spans="1:9">
-      <c r="A30" s="372"/>
-      <c r="B30" s="373"/>
-      <c r="C30" s="373"/>
-      <c r="D30" s="373"/>
-      <c r="E30" s="373"/>
-      <c r="F30" s="373"/>
-      <c r="G30" s="373"/>
-      <c r="H30" s="373"/>
-      <c r="I30" s="374"/>
+      <c r="A30" s="368"/>
+      <c r="B30" s="369"/>
+      <c r="C30" s="369"/>
+      <c r="D30" s="369"/>
+      <c r="E30" s="369"/>
+      <c r="F30" s="369"/>
+      <c r="G30" s="369"/>
+      <c r="H30" s="369"/>
+      <c r="I30" s="370"/>
     </row>
     <row r="31" spans="1:9">
-      <c r="A31" s="372"/>
-      <c r="B31" s="373"/>
-      <c r="C31" s="373"/>
-      <c r="D31" s="373"/>
-      <c r="E31" s="373"/>
-      <c r="F31" s="373"/>
-      <c r="G31" s="373"/>
-      <c r="H31" s="373"/>
-      <c r="I31" s="374"/>
+      <c r="A31" s="368"/>
+      <c r="B31" s="369"/>
+      <c r="C31" s="369"/>
+      <c r="D31" s="369"/>
+      <c r="E31" s="369"/>
+      <c r="F31" s="369"/>
+      <c r="G31" s="369"/>
+      <c r="H31" s="369"/>
+      <c r="I31" s="370"/>
     </row>
     <row r="32" spans="1:9">
-      <c r="A32" s="372"/>
-      <c r="B32" s="373"/>
-      <c r="C32" s="373"/>
-      <c r="D32" s="373"/>
-      <c r="E32" s="373"/>
-      <c r="F32" s="373"/>
-      <c r="G32" s="373"/>
-      <c r="H32" s="373"/>
-      <c r="I32" s="374"/>
+      <c r="A32" s="368"/>
+      <c r="B32" s="369"/>
+      <c r="C32" s="369"/>
+      <c r="D32" s="369"/>
+      <c r="E32" s="369"/>
+      <c r="F32" s="369"/>
+      <c r="G32" s="369"/>
+      <c r="H32" s="369"/>
+      <c r="I32" s="370"/>
     </row>
     <row r="33" spans="1:9">
-      <c r="A33" s="372"/>
-      <c r="B33" s="373"/>
-      <c r="C33" s="373"/>
-      <c r="D33" s="373"/>
-      <c r="E33" s="373"/>
-      <c r="F33" s="373"/>
-      <c r="G33" s="373"/>
-      <c r="H33" s="373"/>
-      <c r="I33" s="374"/>
+      <c r="A33" s="368"/>
+      <c r="B33" s="369"/>
+      <c r="C33" s="369"/>
+      <c r="D33" s="369"/>
+      <c r="E33" s="369"/>
+      <c r="F33" s="369"/>
+      <c r="G33" s="369"/>
+      <c r="H33" s="369"/>
+      <c r="I33" s="370"/>
     </row>
     <row r="34" spans="1:9">
-      <c r="A34" s="372"/>
-      <c r="B34" s="373"/>
-      <c r="C34" s="373"/>
-      <c r="D34" s="373"/>
-      <c r="E34" s="373"/>
-      <c r="F34" s="373"/>
-      <c r="G34" s="373"/>
-      <c r="H34" s="373"/>
-      <c r="I34" s="374"/>
+      <c r="A34" s="368"/>
+      <c r="B34" s="369"/>
+      <c r="C34" s="369"/>
+      <c r="D34" s="369"/>
+      <c r="E34" s="369"/>
+      <c r="F34" s="369"/>
+      <c r="G34" s="369"/>
+      <c r="H34" s="369"/>
+      <c r="I34" s="370"/>
     </row>
     <row r="35" spans="1:9">
-      <c r="A35" s="372"/>
-      <c r="B35" s="373"/>
-      <c r="C35" s="373"/>
-      <c r="D35" s="373"/>
-      <c r="E35" s="373"/>
-      <c r="F35" s="373"/>
-      <c r="G35" s="373"/>
-      <c r="H35" s="373"/>
-      <c r="I35" s="374"/>
+      <c r="A35" s="368"/>
+      <c r="B35" s="369"/>
+      <c r="C35" s="369"/>
+      <c r="D35" s="369"/>
+      <c r="E35" s="369"/>
+      <c r="F35" s="369"/>
+      <c r="G35" s="369"/>
+      <c r="H35" s="369"/>
+      <c r="I35" s="370"/>
     </row>
     <row r="36" spans="1:9">
-      <c r="A36" s="372"/>
-      <c r="B36" s="373"/>
-      <c r="C36" s="373"/>
-      <c r="D36" s="373"/>
-      <c r="E36" s="373"/>
-      <c r="F36" s="373"/>
-      <c r="G36" s="373"/>
-      <c r="H36" s="373"/>
-      <c r="I36" s="374"/>
+      <c r="A36" s="368"/>
+      <c r="B36" s="369"/>
+      <c r="C36" s="369"/>
+      <c r="D36" s="369"/>
+      <c r="E36" s="369"/>
+      <c r="F36" s="369"/>
+      <c r="G36" s="369"/>
+      <c r="H36" s="369"/>
+      <c r="I36" s="370"/>
     </row>
     <row r="37" spans="1:9">
-      <c r="A37" s="372"/>
-      <c r="B37" s="373"/>
-      <c r="C37" s="373"/>
-      <c r="D37" s="373"/>
-      <c r="E37" s="373"/>
-      <c r="F37" s="373"/>
-      <c r="G37" s="373"/>
-      <c r="H37" s="373"/>
-      <c r="I37" s="374"/>
+      <c r="A37" s="368"/>
+      <c r="B37" s="369"/>
+      <c r="C37" s="369"/>
+      <c r="D37" s="369"/>
+      <c r="E37" s="369"/>
+      <c r="F37" s="369"/>
+      <c r="G37" s="369"/>
+      <c r="H37" s="369"/>
+      <c r="I37" s="370"/>
     </row>
     <row r="38" spans="1:9">
-      <c r="A38" s="372"/>
-      <c r="B38" s="373"/>
-      <c r="C38" s="373"/>
-      <c r="D38" s="373"/>
-      <c r="E38" s="373"/>
-      <c r="F38" s="373"/>
-      <c r="G38" s="373"/>
-      <c r="H38" s="373"/>
-      <c r="I38" s="374"/>
+      <c r="A38" s="368"/>
+      <c r="B38" s="369"/>
+      <c r="C38" s="369"/>
+      <c r="D38" s="369"/>
+      <c r="E38" s="369"/>
+      <c r="F38" s="369"/>
+      <c r="G38" s="369"/>
+      <c r="H38" s="369"/>
+      <c r="I38" s="370"/>
     </row>
     <row r="39" spans="1:9">
-      <c r="A39" s="372"/>
-      <c r="B39" s="373"/>
-      <c r="C39" s="373"/>
-      <c r="D39" s="373"/>
-      <c r="E39" s="373"/>
-      <c r="F39" s="373"/>
-      <c r="G39" s="373"/>
-      <c r="H39" s="373"/>
-      <c r="I39" s="374"/>
+      <c r="A39" s="368"/>
+      <c r="B39" s="369"/>
+      <c r="C39" s="369"/>
+      <c r="D39" s="369"/>
+      <c r="E39" s="369"/>
+      <c r="F39" s="369"/>
+      <c r="G39" s="369"/>
+      <c r="H39" s="369"/>
+      <c r="I39" s="370"/>
     </row>
     <row r="40" spans="1:9">
-      <c r="A40" s="372"/>
-      <c r="B40" s="373"/>
-      <c r="C40" s="373"/>
-      <c r="D40" s="373"/>
-      <c r="E40" s="373"/>
-      <c r="F40" s="373"/>
-      <c r="G40" s="373"/>
-      <c r="H40" s="373"/>
-      <c r="I40" s="374"/>
+      <c r="A40" s="368"/>
+      <c r="B40" s="369"/>
+      <c r="C40" s="369"/>
+      <c r="D40" s="369"/>
+      <c r="E40" s="369"/>
+      <c r="F40" s="369"/>
+      <c r="G40" s="369"/>
+      <c r="H40" s="369"/>
+      <c r="I40" s="370"/>
     </row>
     <row r="41" spans="1:9">
-      <c r="A41" s="375"/>
-      <c r="B41" s="376"/>
-      <c r="C41" s="376"/>
-      <c r="D41" s="376"/>
-      <c r="E41" s="376"/>
-      <c r="F41" s="376"/>
-      <c r="G41" s="376"/>
-      <c r="H41" s="376"/>
-      <c r="I41" s="377"/>
+      <c r="A41" s="371"/>
+      <c r="B41" s="372"/>
+      <c r="C41" s="372"/>
+      <c r="D41" s="372"/>
+      <c r="E41" s="372"/>
+      <c r="F41" s="372"/>
+      <c r="G41" s="372"/>
+      <c r="H41" s="372"/>
+      <c r="I41" s="373"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -36977,7 +36954,7 @@
       <c r="H4" s="93"/>
     </row>
     <row r="5" spans="1:10" ht="15.75" customHeight="1">
-      <c r="F5" s="365" t="s">
+      <c r="F5" s="404" t="s">
         <v>82</v>
       </c>
       <c r="G5" s="407"/>
@@ -38186,76 +38163,76 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:14" ht="35.25" customHeight="1">
-      <c r="A1" s="408" t="s">
+      <c r="A1" s="410" t="s">
         <v>598</v>
       </c>
-      <c r="B1" s="408"/>
-      <c r="C1" s="408"/>
-      <c r="D1" s="408"/>
-      <c r="E1" s="408"/>
-      <c r="F1" s="408"/>
-      <c r="G1" s="408"/>
-      <c r="H1" s="408"/>
-      <c r="I1" s="408"/>
-      <c r="J1" s="408"/>
-      <c r="K1" s="408"/>
-      <c r="L1" s="408"/>
-      <c r="M1" s="408"/>
-      <c r="N1" s="408"/>
+      <c r="B1" s="410"/>
+      <c r="C1" s="410"/>
+      <c r="D1" s="410"/>
+      <c r="E1" s="410"/>
+      <c r="F1" s="410"/>
+      <c r="G1" s="410"/>
+      <c r="H1" s="410"/>
+      <c r="I1" s="410"/>
+      <c r="J1" s="410"/>
+      <c r="K1" s="410"/>
+      <c r="L1" s="410"/>
+      <c r="M1" s="410"/>
+      <c r="N1" s="410"/>
     </row>
     <row r="3" spans="1:14" ht="50.1" customHeight="1">
-      <c r="A3" s="409" t="s">
+      <c r="A3" s="411" t="s">
         <v>654</v>
       </c>
-      <c r="B3" s="409"/>
-      <c r="C3" s="409"/>
-      <c r="D3" s="409"/>
-      <c r="E3" s="409"/>
-      <c r="F3" s="409"/>
-      <c r="G3" s="409"/>
-      <c r="H3" s="409"/>
-      <c r="I3" s="409"/>
-      <c r="J3" s="409"/>
-      <c r="K3" s="409"/>
-      <c r="L3" s="409"/>
-      <c r="M3" s="409"/>
-      <c r="N3" s="409"/>
+      <c r="B3" s="411"/>
+      <c r="C3" s="411"/>
+      <c r="D3" s="411"/>
+      <c r="E3" s="411"/>
+      <c r="F3" s="411"/>
+      <c r="G3" s="411"/>
+      <c r="H3" s="411"/>
+      <c r="I3" s="411"/>
+      <c r="J3" s="411"/>
+      <c r="K3" s="411"/>
+      <c r="L3" s="411"/>
+      <c r="M3" s="411"/>
+      <c r="N3" s="411"/>
     </row>
     <row r="7" spans="1:14" ht="34.5" customHeight="1">
-      <c r="A7" s="410" t="s">
+      <c r="A7" s="412" t="s">
         <v>599</v>
       </c>
-      <c r="B7" s="410"/>
-      <c r="C7" s="410"/>
-      <c r="D7" s="410"/>
-      <c r="E7" s="410"/>
-      <c r="F7" s="410"/>
-      <c r="G7" s="410"/>
-      <c r="H7" s="410"/>
-      <c r="I7" s="410"/>
-      <c r="J7" s="410"/>
-      <c r="K7" s="410"/>
-      <c r="L7" s="410"/>
-      <c r="M7" s="410"/>
-      <c r="N7" s="410"/>
+      <c r="B7" s="412"/>
+      <c r="C7" s="412"/>
+      <c r="D7" s="412"/>
+      <c r="E7" s="412"/>
+      <c r="F7" s="412"/>
+      <c r="G7" s="412"/>
+      <c r="H7" s="412"/>
+      <c r="I7" s="412"/>
+      <c r="J7" s="412"/>
+      <c r="K7" s="412"/>
+      <c r="L7" s="412"/>
+      <c r="M7" s="412"/>
+      <c r="N7" s="412"/>
     </row>
     <row r="9" spans="1:14" ht="50.1" customHeight="1">
-      <c r="A9" s="409" t="s">
+      <c r="A9" s="411" t="s">
         <v>654</v>
       </c>
-      <c r="B9" s="409"/>
-      <c r="C9" s="409"/>
-      <c r="D9" s="409"/>
-      <c r="E9" s="409"/>
-      <c r="F9" s="409"/>
-      <c r="G9" s="409"/>
-      <c r="H9" s="409"/>
-      <c r="I9" s="409"/>
-      <c r="J9" s="409"/>
-      <c r="K9" s="409"/>
-      <c r="L9" s="409"/>
-      <c r="M9" s="409"/>
-      <c r="N9" s="409"/>
+      <c r="B9" s="411"/>
+      <c r="C9" s="411"/>
+      <c r="D9" s="411"/>
+      <c r="E9" s="411"/>
+      <c r="F9" s="411"/>
+      <c r="G9" s="411"/>
+      <c r="H9" s="411"/>
+      <c r="I9" s="411"/>
+      <c r="J9" s="411"/>
+      <c r="K9" s="411"/>
+      <c r="L9" s="411"/>
+      <c r="M9" s="411"/>
+      <c r="N9" s="411"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -38283,12 +38260,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" s="214" customFormat="1" ht="18" customHeight="1">
-      <c r="A1" s="410" t="s">
+      <c r="A1" s="412" t="s">
         <v>567</v>
       </c>
-      <c r="B1" s="413"/>
-      <c r="C1" s="413"/>
-      <c r="D1" s="413"/>
+      <c r="B1" s="415"/>
+      <c r="C1" s="415"/>
+      <c r="D1" s="415"/>
       <c r="E1" s="362"/>
       <c r="F1" s="362"/>
       <c r="G1" s="362"/>
@@ -38444,18 +38421,18 @@
     </row>
     <row r="20" spans="1:3" ht="15" customHeight="1"/>
     <row r="21" spans="1:3" ht="15" customHeight="1">
-      <c r="A21" s="411" t="s">
+      <c r="A21" s="413" t="s">
         <v>658</v>
       </c>
-      <c r="B21" s="411"/>
-      <c r="C21" s="411"/>
+      <c r="B21" s="413"/>
+      <c r="C21" s="413"/>
     </row>
     <row r="22" spans="1:3" ht="15" customHeight="1">
-      <c r="A22" s="412" t="s">
+      <c r="A22" s="414" t="s">
         <v>516</v>
       </c>
-      <c r="B22" s="412"/>
-      <c r="C22" s="412"/>
+      <c r="B22" s="414"/>
+      <c r="C22" s="414"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -41165,13 +41142,13 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3" ht="45">
-      <c r="A1" s="415" t="s">
+      <c r="A1" s="364" t="s">
         <v>749</v>
       </c>
-      <c r="B1" s="415" t="s">
+      <c r="B1" s="364" t="s">
         <v>750</v>
       </c>
-      <c r="C1" s="415" t="s">
+      <c r="C1" s="364" t="s">
         <v>751</v>
       </c>
     </row>
@@ -41182,7 +41159,7 @@
       <c r="B2" s="292" t="s">
         <v>753</v>
       </c>
-      <c r="C2" s="414" t="s">
+      <c r="C2" s="363" t="s">
         <v>754</v>
       </c>
     </row>
@@ -41193,7 +41170,7 @@
       <c r="B3" s="292" t="s">
         <v>756</v>
       </c>
-      <c r="C3" s="414" t="s">
+      <c r="C3" s="363" t="s">
         <v>757</v>
       </c>
     </row>
@@ -41204,7 +41181,7 @@
       <c r="B4" s="292" t="s">
         <v>759</v>
       </c>
-      <c r="C4" s="414" t="s">
+      <c r="C4" s="363" t="s">
         <v>760</v>
       </c>
     </row>
@@ -41215,7 +41192,7 @@
       <c r="B5" s="292" t="s">
         <v>762</v>
       </c>
-      <c r="C5" s="414" t="s">
+      <c r="C5" s="363" t="s">
         <v>763</v>
       </c>
     </row>
@@ -41226,7 +41203,7 @@
       <c r="B6" s="292" t="s">
         <v>765</v>
       </c>
-      <c r="C6" s="414" t="s">
+      <c r="C6" s="363" t="s">
         <v>766</v>
       </c>
     </row>
@@ -41234,10 +41211,10 @@
       <c r="A7" s="292" t="s">
         <v>767</v>
       </c>
-      <c r="B7" s="414" t="s">
+      <c r="B7" s="363" t="s">
         <v>768</v>
       </c>
-      <c r="C7" s="414" t="s">
+      <c r="C7" s="363" t="s">
         <v>769</v>
       </c>
     </row>
@@ -42723,244 +42700,244 @@
       <c r="O64" s="2"/>
     </row>
     <row r="65" spans="1:24" s="74" customFormat="1" ht="18.75" customHeight="1">
-      <c r="A65" s="381" t="s">
+      <c r="A65" s="377" t="s">
         <v>500</v>
       </c>
-      <c r="B65" s="381"/>
-      <c r="C65" s="381"/>
-      <c r="D65" s="381"/>
-      <c r="E65" s="381"/>
-      <c r="F65" s="381"/>
-      <c r="G65" s="381"/>
-      <c r="H65" s="381"/>
-      <c r="I65" s="381"/>
-      <c r="J65" s="381"/>
-      <c r="K65" s="381"/>
-      <c r="L65" s="381"/>
-      <c r="M65" s="381"/>
-      <c r="N65" s="381"/>
-      <c r="O65" s="381"/>
-      <c r="P65" s="381"/>
-      <c r="Q65" s="381"/>
-      <c r="R65" s="381"/>
-      <c r="S65" s="381"/>
-      <c r="T65" s="381"/>
+      <c r="B65" s="377"/>
+      <c r="C65" s="377"/>
+      <c r="D65" s="377"/>
+      <c r="E65" s="377"/>
+      <c r="F65" s="377"/>
+      <c r="G65" s="377"/>
+      <c r="H65" s="377"/>
+      <c r="I65" s="377"/>
+      <c r="J65" s="377"/>
+      <c r="K65" s="377"/>
+      <c r="L65" s="377"/>
+      <c r="M65" s="377"/>
+      <c r="N65" s="377"/>
+      <c r="O65" s="377"/>
+      <c r="P65" s="377"/>
+      <c r="Q65" s="377"/>
+      <c r="R65" s="377"/>
+      <c r="S65" s="377"/>
+      <c r="T65" s="377"/>
       <c r="U65" s="170"/>
       <c r="V65" s="170"/>
       <c r="W65" s="170"/>
       <c r="X65" s="170"/>
     </row>
     <row r="66" spans="1:24" s="170" customFormat="1" ht="18.75" customHeight="1">
-      <c r="A66" s="381" t="s">
+      <c r="A66" s="377" t="s">
         <v>501</v>
       </c>
-      <c r="B66" s="381"/>
-      <c r="C66" s="381"/>
-      <c r="D66" s="381"/>
-      <c r="E66" s="381"/>
-      <c r="F66" s="381"/>
-      <c r="G66" s="381"/>
-      <c r="H66" s="381"/>
-      <c r="I66" s="381"/>
-      <c r="J66" s="381"/>
-      <c r="K66" s="381"/>
-      <c r="L66" s="381"/>
-      <c r="M66" s="381"/>
-      <c r="N66" s="381"/>
-      <c r="O66" s="381"/>
-      <c r="P66" s="381"/>
-      <c r="Q66" s="381"/>
-      <c r="R66" s="381"/>
-      <c r="S66" s="381"/>
-      <c r="T66" s="381"/>
+      <c r="B66" s="377"/>
+      <c r="C66" s="377"/>
+      <c r="D66" s="377"/>
+      <c r="E66" s="377"/>
+      <c r="F66" s="377"/>
+      <c r="G66" s="377"/>
+      <c r="H66" s="377"/>
+      <c r="I66" s="377"/>
+      <c r="J66" s="377"/>
+      <c r="K66" s="377"/>
+      <c r="L66" s="377"/>
+      <c r="M66" s="377"/>
+      <c r="N66" s="377"/>
+      <c r="O66" s="377"/>
+      <c r="P66" s="377"/>
+      <c r="Q66" s="377"/>
+      <c r="R66" s="377"/>
+      <c r="S66" s="377"/>
+      <c r="T66" s="377"/>
     </row>
     <row r="67" spans="1:24" customFormat="1" ht="30.75" customHeight="1">
-      <c r="A67" s="382" t="s">
+      <c r="A67" s="378" t="s">
         <v>736</v>
       </c>
-      <c r="B67" s="382"/>
-      <c r="C67" s="382"/>
-      <c r="D67" s="382"/>
-      <c r="E67" s="382"/>
-      <c r="F67" s="382"/>
-      <c r="G67" s="382"/>
-      <c r="H67" s="382"/>
-      <c r="I67" s="382"/>
-      <c r="J67" s="382"/>
-      <c r="K67" s="382"/>
-      <c r="L67" s="382"/>
-      <c r="M67" s="382"/>
-      <c r="N67" s="382"/>
-      <c r="O67" s="382"/>
-      <c r="P67" s="382"/>
-      <c r="Q67" s="382"/>
-      <c r="R67" s="382"/>
-      <c r="S67" s="382"/>
-      <c r="T67" s="382"/>
+      <c r="B67" s="378"/>
+      <c r="C67" s="378"/>
+      <c r="D67" s="378"/>
+      <c r="E67" s="378"/>
+      <c r="F67" s="378"/>
+      <c r="G67" s="378"/>
+      <c r="H67" s="378"/>
+      <c r="I67" s="378"/>
+      <c r="J67" s="378"/>
+      <c r="K67" s="378"/>
+      <c r="L67" s="378"/>
+      <c r="M67" s="378"/>
+      <c r="N67" s="378"/>
+      <c r="O67" s="378"/>
+      <c r="P67" s="378"/>
+      <c r="Q67" s="378"/>
+      <c r="R67" s="378"/>
+      <c r="S67" s="378"/>
+      <c r="T67" s="378"/>
       <c r="U67" s="22"/>
       <c r="V67" s="22"/>
       <c r="W67" s="22"/>
       <c r="X67" s="1"/>
     </row>
     <row r="68" spans="1:24" customFormat="1" ht="30.75" customHeight="1">
-      <c r="A68" s="382" t="s">
+      <c r="A68" s="378" t="s">
         <v>502</v>
       </c>
-      <c r="B68" s="382"/>
-      <c r="C68" s="382"/>
-      <c r="D68" s="382"/>
-      <c r="E68" s="382"/>
-      <c r="F68" s="382"/>
-      <c r="G68" s="382"/>
-      <c r="H68" s="382"/>
-      <c r="I68" s="382"/>
-      <c r="J68" s="382"/>
-      <c r="K68" s="382"/>
-      <c r="L68" s="382"/>
-      <c r="M68" s="382"/>
-      <c r="N68" s="382"/>
-      <c r="O68" s="382"/>
-      <c r="P68" s="382"/>
-      <c r="Q68" s="382"/>
-      <c r="R68" s="382"/>
-      <c r="S68" s="382"/>
-      <c r="T68" s="382"/>
+      <c r="B68" s="378"/>
+      <c r="C68" s="378"/>
+      <c r="D68" s="378"/>
+      <c r="E68" s="378"/>
+      <c r="F68" s="378"/>
+      <c r="G68" s="378"/>
+      <c r="H68" s="378"/>
+      <c r="I68" s="378"/>
+      <c r="J68" s="378"/>
+      <c r="K68" s="378"/>
+      <c r="L68" s="378"/>
+      <c r="M68" s="378"/>
+      <c r="N68" s="378"/>
+      <c r="O68" s="378"/>
+      <c r="P68" s="378"/>
+      <c r="Q68" s="378"/>
+      <c r="R68" s="378"/>
+      <c r="S68" s="378"/>
+      <c r="T68" s="378"/>
       <c r="U68" s="22"/>
       <c r="V68" s="22"/>
       <c r="W68" s="22"/>
       <c r="X68" s="1"/>
     </row>
     <row r="69" spans="1:24" s="170" customFormat="1" ht="18.75" customHeight="1">
-      <c r="A69" s="383" t="s">
+      <c r="A69" s="379" t="s">
         <v>503</v>
       </c>
-      <c r="B69" s="383"/>
-      <c r="C69" s="383"/>
-      <c r="D69" s="383"/>
-      <c r="E69" s="383"/>
-      <c r="F69" s="383"/>
-      <c r="G69" s="383"/>
-      <c r="H69" s="383"/>
-      <c r="I69" s="383"/>
-      <c r="J69" s="383"/>
-      <c r="K69" s="383"/>
-      <c r="L69" s="383"/>
-      <c r="M69" s="383"/>
-      <c r="N69" s="383"/>
-      <c r="O69" s="383"/>
-      <c r="P69" s="383"/>
-      <c r="Q69" s="383"/>
-      <c r="R69" s="383"/>
-      <c r="S69" s="383"/>
-      <c r="T69" s="383"/>
+      <c r="B69" s="379"/>
+      <c r="C69" s="379"/>
+      <c r="D69" s="379"/>
+      <c r="E69" s="379"/>
+      <c r="F69" s="379"/>
+      <c r="G69" s="379"/>
+      <c r="H69" s="379"/>
+      <c r="I69" s="379"/>
+      <c r="J69" s="379"/>
+      <c r="K69" s="379"/>
+      <c r="L69" s="379"/>
+      <c r="M69" s="379"/>
+      <c r="N69" s="379"/>
+      <c r="O69" s="379"/>
+      <c r="P69" s="379"/>
+      <c r="Q69" s="379"/>
+      <c r="R69" s="379"/>
+      <c r="S69" s="379"/>
+      <c r="T69" s="379"/>
       <c r="U69" s="44"/>
       <c r="V69" s="44"/>
       <c r="W69" s="44"/>
       <c r="X69" s="74"/>
     </row>
     <row r="70" spans="1:24" customFormat="1" ht="30.75" customHeight="1">
-      <c r="A70" s="380" t="s">
+      <c r="A70" s="376" t="s">
         <v>676</v>
       </c>
-      <c r="B70" s="380"/>
-      <c r="C70" s="380"/>
-      <c r="D70" s="380"/>
-      <c r="E70" s="380"/>
-      <c r="F70" s="380"/>
-      <c r="G70" s="380"/>
-      <c r="H70" s="380"/>
-      <c r="I70" s="380"/>
-      <c r="J70" s="380"/>
-      <c r="K70" s="380"/>
-      <c r="L70" s="380"/>
-      <c r="M70" s="380"/>
-      <c r="N70" s="380"/>
-      <c r="O70" s="380"/>
-      <c r="P70" s="380"/>
-      <c r="Q70" s="380"/>
-      <c r="R70" s="380"/>
-      <c r="S70" s="380"/>
-      <c r="T70" s="380"/>
+      <c r="B70" s="376"/>
+      <c r="C70" s="376"/>
+      <c r="D70" s="376"/>
+      <c r="E70" s="376"/>
+      <c r="F70" s="376"/>
+      <c r="G70" s="376"/>
+      <c r="H70" s="376"/>
+      <c r="I70" s="376"/>
+      <c r="J70" s="376"/>
+      <c r="K70" s="376"/>
+      <c r="L70" s="376"/>
+      <c r="M70" s="376"/>
+      <c r="N70" s="376"/>
+      <c r="O70" s="376"/>
+      <c r="P70" s="376"/>
+      <c r="Q70" s="376"/>
+      <c r="R70" s="376"/>
+      <c r="S70" s="376"/>
+      <c r="T70" s="376"/>
       <c r="U70" s="22"/>
       <c r="V70" s="22"/>
       <c r="W70" s="22"/>
       <c r="X70" s="1"/>
     </row>
     <row r="71" spans="1:24" s="170" customFormat="1" ht="18.75" customHeight="1">
-      <c r="A71" s="379" t="s">
+      <c r="A71" s="375" t="s">
         <v>504</v>
       </c>
-      <c r="B71" s="379"/>
-      <c r="C71" s="379"/>
-      <c r="D71" s="379"/>
-      <c r="E71" s="379"/>
-      <c r="F71" s="379"/>
-      <c r="G71" s="379"/>
-      <c r="H71" s="379"/>
-      <c r="I71" s="379"/>
-      <c r="J71" s="379"/>
-      <c r="K71" s="379"/>
-      <c r="L71" s="379"/>
-      <c r="M71" s="379"/>
-      <c r="N71" s="379"/>
-      <c r="O71" s="379"/>
-      <c r="P71" s="379"/>
-      <c r="Q71" s="379"/>
-      <c r="R71" s="379"/>
-      <c r="S71" s="379"/>
-      <c r="T71" s="379"/>
+      <c r="B71" s="375"/>
+      <c r="C71" s="375"/>
+      <c r="D71" s="375"/>
+      <c r="E71" s="375"/>
+      <c r="F71" s="375"/>
+      <c r="G71" s="375"/>
+      <c r="H71" s="375"/>
+      <c r="I71" s="375"/>
+      <c r="J71" s="375"/>
+      <c r="K71" s="375"/>
+      <c r="L71" s="375"/>
+      <c r="M71" s="375"/>
+      <c r="N71" s="375"/>
+      <c r="O71" s="375"/>
+      <c r="P71" s="375"/>
+      <c r="Q71" s="375"/>
+      <c r="R71" s="375"/>
+      <c r="S71" s="375"/>
+      <c r="T71" s="375"/>
     </row>
     <row r="72" spans="1:24" s="170" customFormat="1" ht="18.75" customHeight="1">
-      <c r="A72" s="379" t="s">
+      <c r="A72" s="375" t="s">
         <v>505</v>
       </c>
-      <c r="B72" s="379"/>
-      <c r="C72" s="379"/>
-      <c r="D72" s="379"/>
-      <c r="E72" s="379"/>
-      <c r="F72" s="379"/>
-      <c r="G72" s="379"/>
-      <c r="H72" s="379"/>
-      <c r="I72" s="379"/>
-      <c r="J72" s="379"/>
-      <c r="K72" s="379"/>
-      <c r="L72" s="379"/>
-      <c r="M72" s="379"/>
-      <c r="N72" s="379"/>
-      <c r="O72" s="379"/>
-      <c r="P72" s="379"/>
-      <c r="Q72" s="379"/>
-      <c r="R72" s="379"/>
-      <c r="S72" s="379"/>
-      <c r="T72" s="379"/>
+      <c r="B72" s="375"/>
+      <c r="C72" s="375"/>
+      <c r="D72" s="375"/>
+      <c r="E72" s="375"/>
+      <c r="F72" s="375"/>
+      <c r="G72" s="375"/>
+      <c r="H72" s="375"/>
+      <c r="I72" s="375"/>
+      <c r="J72" s="375"/>
+      <c r="K72" s="375"/>
+      <c r="L72" s="375"/>
+      <c r="M72" s="375"/>
+      <c r="N72" s="375"/>
+      <c r="O72" s="375"/>
+      <c r="P72" s="375"/>
+      <c r="Q72" s="375"/>
+      <c r="R72" s="375"/>
+      <c r="S72" s="375"/>
+      <c r="T72" s="375"/>
       <c r="U72" s="74"/>
       <c r="V72" s="74"/>
       <c r="W72" s="74"/>
       <c r="X72" s="74"/>
     </row>
     <row r="73" spans="1:24" s="170" customFormat="1" ht="18.75" customHeight="1">
-      <c r="A73" s="378" t="s">
+      <c r="A73" s="374" t="s">
         <v>660</v>
       </c>
-      <c r="B73" s="378"/>
-      <c r="C73" s="378"/>
-      <c r="D73" s="378"/>
-      <c r="E73" s="378"/>
-      <c r="F73" s="378"/>
-      <c r="G73" s="378"/>
-      <c r="H73" s="378"/>
-      <c r="I73" s="378"/>
-      <c r="J73" s="378"/>
-      <c r="K73" s="378"/>
-      <c r="L73" s="378"/>
-      <c r="M73" s="378"/>
-      <c r="N73" s="378"/>
-      <c r="O73" s="378"/>
-      <c r="P73" s="378"/>
-      <c r="Q73" s="378"/>
-      <c r="R73" s="378"/>
-      <c r="S73" s="378"/>
-      <c r="T73" s="378"/>
+      <c r="B73" s="374"/>
+      <c r="C73" s="374"/>
+      <c r="D73" s="374"/>
+      <c r="E73" s="374"/>
+      <c r="F73" s="374"/>
+      <c r="G73" s="374"/>
+      <c r="H73" s="374"/>
+      <c r="I73" s="374"/>
+      <c r="J73" s="374"/>
+      <c r="K73" s="374"/>
+      <c r="L73" s="374"/>
+      <c r="M73" s="374"/>
+      <c r="N73" s="374"/>
+      <c r="O73" s="374"/>
+      <c r="P73" s="374"/>
+      <c r="Q73" s="374"/>
+      <c r="R73" s="374"/>
+      <c r="S73" s="374"/>
+      <c r="T73" s="374"/>
       <c r="U73" s="74"/>
       <c r="V73" s="74"/>
       <c r="W73" s="74"/>
@@ -43722,316 +43699,316 @@
       <c r="O28" s="2"/>
     </row>
     <row r="29" spans="1:18" ht="30.75" customHeight="1">
-      <c r="A29" s="385" t="s">
+      <c r="A29" s="381" t="s">
         <v>641</v>
       </c>
-      <c r="B29" s="387"/>
-      <c r="C29" s="387"/>
-      <c r="D29" s="387"/>
-      <c r="E29" s="387"/>
-      <c r="F29" s="387"/>
-      <c r="G29" s="387"/>
-      <c r="H29" s="387"/>
-      <c r="I29" s="387"/>
-      <c r="J29" s="387"/>
-      <c r="K29" s="387"/>
-      <c r="L29" s="387"/>
-      <c r="M29" s="387"/>
-      <c r="N29" s="387"/>
-      <c r="O29" s="387"/>
-      <c r="P29" s="387"/>
-      <c r="Q29" s="387"/>
-      <c r="R29" s="386"/>
+      <c r="B29" s="383"/>
+      <c r="C29" s="383"/>
+      <c r="D29" s="383"/>
+      <c r="E29" s="383"/>
+      <c r="F29" s="383"/>
+      <c r="G29" s="383"/>
+      <c r="H29" s="383"/>
+      <c r="I29" s="383"/>
+      <c r="J29" s="383"/>
+      <c r="K29" s="383"/>
+      <c r="L29" s="383"/>
+      <c r="M29" s="383"/>
+      <c r="N29" s="383"/>
+      <c r="O29" s="383"/>
+      <c r="P29" s="383"/>
+      <c r="Q29" s="383"/>
+      <c r="R29" s="382"/>
     </row>
     <row r="30" spans="1:18" ht="18.75" customHeight="1">
-      <c r="A30" s="385" t="s">
+      <c r="A30" s="381" t="s">
         <v>506</v>
       </c>
-      <c r="B30" s="387"/>
-      <c r="C30" s="387"/>
-      <c r="D30" s="387"/>
-      <c r="E30" s="387"/>
-      <c r="F30" s="387"/>
-      <c r="G30" s="387"/>
-      <c r="H30" s="387"/>
-      <c r="I30" s="387"/>
-      <c r="J30" s="387"/>
-      <c r="K30" s="387"/>
-      <c r="L30" s="387"/>
-      <c r="M30" s="387"/>
-      <c r="N30" s="387"/>
-      <c r="O30" s="387"/>
-      <c r="P30" s="387"/>
-      <c r="Q30" s="387"/>
-      <c r="R30" s="386"/>
+      <c r="B30" s="383"/>
+      <c r="C30" s="383"/>
+      <c r="D30" s="383"/>
+      <c r="E30" s="383"/>
+      <c r="F30" s="383"/>
+      <c r="G30" s="383"/>
+      <c r="H30" s="383"/>
+      <c r="I30" s="383"/>
+      <c r="J30" s="383"/>
+      <c r="K30" s="383"/>
+      <c r="L30" s="383"/>
+      <c r="M30" s="383"/>
+      <c r="N30" s="383"/>
+      <c r="O30" s="383"/>
+      <c r="P30" s="383"/>
+      <c r="Q30" s="383"/>
+      <c r="R30" s="382"/>
     </row>
     <row r="31" spans="1:18" ht="18.75" customHeight="1">
-      <c r="A31" s="385" t="s">
+      <c r="A31" s="381" t="s">
         <v>507</v>
       </c>
-      <c r="B31" s="386"/>
-      <c r="C31" s="386"/>
-      <c r="D31" s="386"/>
-      <c r="E31" s="386"/>
-      <c r="F31" s="386"/>
-      <c r="G31" s="386"/>
-      <c r="H31" s="386"/>
-      <c r="I31" s="386"/>
-      <c r="J31" s="386"/>
-      <c r="K31" s="386"/>
-      <c r="L31" s="386"/>
-      <c r="M31" s="386"/>
-      <c r="N31" s="386"/>
-      <c r="O31" s="386"/>
-      <c r="P31" s="386"/>
-      <c r="Q31" s="386"/>
-      <c r="R31" s="386"/>
+      <c r="B31" s="382"/>
+      <c r="C31" s="382"/>
+      <c r="D31" s="382"/>
+      <c r="E31" s="382"/>
+      <c r="F31" s="382"/>
+      <c r="G31" s="382"/>
+      <c r="H31" s="382"/>
+      <c r="I31" s="382"/>
+      <c r="J31" s="382"/>
+      <c r="K31" s="382"/>
+      <c r="L31" s="382"/>
+      <c r="M31" s="382"/>
+      <c r="N31" s="382"/>
+      <c r="O31" s="382"/>
+      <c r="P31" s="382"/>
+      <c r="Q31" s="382"/>
+      <c r="R31" s="382"/>
     </row>
     <row r="32" spans="1:18" ht="30.75" customHeight="1">
-      <c r="A32" s="385" t="s">
+      <c r="A32" s="381" t="s">
         <v>667</v>
       </c>
-      <c r="B32" s="386"/>
-      <c r="C32" s="386"/>
-      <c r="D32" s="386"/>
-      <c r="E32" s="386"/>
-      <c r="F32" s="386"/>
-      <c r="G32" s="386"/>
-      <c r="H32" s="386"/>
-      <c r="I32" s="386"/>
-      <c r="J32" s="386"/>
-      <c r="K32" s="386"/>
-      <c r="L32" s="386"/>
-      <c r="M32" s="386"/>
-      <c r="N32" s="386"/>
-      <c r="O32" s="386"/>
-      <c r="P32" s="386"/>
-      <c r="Q32" s="386"/>
-      <c r="R32" s="386"/>
+      <c r="B32" s="382"/>
+      <c r="C32" s="382"/>
+      <c r="D32" s="382"/>
+      <c r="E32" s="382"/>
+      <c r="F32" s="382"/>
+      <c r="G32" s="382"/>
+      <c r="H32" s="382"/>
+      <c r="I32" s="382"/>
+      <c r="J32" s="382"/>
+      <c r="K32" s="382"/>
+      <c r="L32" s="382"/>
+      <c r="M32" s="382"/>
+      <c r="N32" s="382"/>
+      <c r="O32" s="382"/>
+      <c r="P32" s="382"/>
+      <c r="Q32" s="382"/>
+      <c r="R32" s="382"/>
     </row>
     <row r="33" spans="1:21" ht="18.75" customHeight="1">
-      <c r="A33" s="385" t="s">
+      <c r="A33" s="381" t="s">
         <v>508</v>
       </c>
-      <c r="B33" s="386"/>
-      <c r="C33" s="386"/>
-      <c r="D33" s="386"/>
-      <c r="E33" s="386"/>
-      <c r="F33" s="386"/>
-      <c r="G33" s="386"/>
-      <c r="H33" s="386"/>
-      <c r="I33" s="386"/>
-      <c r="J33" s="386"/>
-      <c r="K33" s="386"/>
-      <c r="L33" s="386"/>
-      <c r="M33" s="386"/>
-      <c r="N33" s="386"/>
-      <c r="O33" s="386"/>
-      <c r="P33" s="386"/>
-      <c r="Q33" s="386"/>
-      <c r="R33" s="386"/>
+      <c r="B33" s="382"/>
+      <c r="C33" s="382"/>
+      <c r="D33" s="382"/>
+      <c r="E33" s="382"/>
+      <c r="F33" s="382"/>
+      <c r="G33" s="382"/>
+      <c r="H33" s="382"/>
+      <c r="I33" s="382"/>
+      <c r="J33" s="382"/>
+      <c r="K33" s="382"/>
+      <c r="L33" s="382"/>
+      <c r="M33" s="382"/>
+      <c r="N33" s="382"/>
+      <c r="O33" s="382"/>
+      <c r="P33" s="382"/>
+      <c r="Q33" s="382"/>
+      <c r="R33" s="382"/>
     </row>
     <row r="34" spans="1:21" ht="30.75" customHeight="1">
-      <c r="A34" s="385" t="s">
+      <c r="A34" s="381" t="s">
         <v>95</v>
       </c>
-      <c r="B34" s="386"/>
-      <c r="C34" s="386"/>
-      <c r="D34" s="386"/>
-      <c r="E34" s="386"/>
-      <c r="F34" s="386"/>
-      <c r="G34" s="386"/>
-      <c r="H34" s="386"/>
-      <c r="I34" s="386"/>
-      <c r="J34" s="386"/>
-      <c r="K34" s="386"/>
-      <c r="L34" s="386"/>
-      <c r="M34" s="386"/>
-      <c r="N34" s="386"/>
-      <c r="O34" s="386"/>
-      <c r="P34" s="386"/>
-      <c r="Q34" s="386"/>
-      <c r="R34" s="386"/>
+      <c r="B34" s="382"/>
+      <c r="C34" s="382"/>
+      <c r="D34" s="382"/>
+      <c r="E34" s="382"/>
+      <c r="F34" s="382"/>
+      <c r="G34" s="382"/>
+      <c r="H34" s="382"/>
+      <c r="I34" s="382"/>
+      <c r="J34" s="382"/>
+      <c r="K34" s="382"/>
+      <c r="L34" s="382"/>
+      <c r="M34" s="382"/>
+      <c r="N34" s="382"/>
+      <c r="O34" s="382"/>
+      <c r="P34" s="382"/>
+      <c r="Q34" s="382"/>
+      <c r="R34" s="382"/>
     </row>
     <row r="35" spans="1:21" ht="18.75" customHeight="1">
-      <c r="A35" s="388" t="s">
+      <c r="A35" s="384" t="s">
         <v>96</v>
       </c>
-      <c r="B35" s="386"/>
-      <c r="C35" s="386"/>
-      <c r="D35" s="386"/>
-      <c r="E35" s="386"/>
-      <c r="F35" s="386"/>
-      <c r="G35" s="386"/>
-      <c r="H35" s="386"/>
-      <c r="I35" s="386"/>
-      <c r="J35" s="386"/>
-      <c r="K35" s="386"/>
-      <c r="L35" s="386"/>
-      <c r="M35" s="386"/>
-      <c r="N35" s="386"/>
-      <c r="O35" s="386"/>
-      <c r="P35" s="386"/>
-      <c r="Q35" s="386"/>
-      <c r="R35" s="386"/>
+      <c r="B35" s="382"/>
+      <c r="C35" s="382"/>
+      <c r="D35" s="382"/>
+      <c r="E35" s="382"/>
+      <c r="F35" s="382"/>
+      <c r="G35" s="382"/>
+      <c r="H35" s="382"/>
+      <c r="I35" s="382"/>
+      <c r="J35" s="382"/>
+      <c r="K35" s="382"/>
+      <c r="L35" s="382"/>
+      <c r="M35" s="382"/>
+      <c r="N35" s="382"/>
+      <c r="O35" s="382"/>
+      <c r="P35" s="382"/>
+      <c r="Q35" s="382"/>
+      <c r="R35" s="382"/>
     </row>
     <row r="36" spans="1:21" ht="30.75" customHeight="1">
-      <c r="A36" s="388" t="s">
+      <c r="A36" s="384" t="s">
         <v>675</v>
       </c>
-      <c r="B36" s="386"/>
-      <c r="C36" s="386"/>
-      <c r="D36" s="386"/>
-      <c r="E36" s="386"/>
-      <c r="F36" s="386"/>
-      <c r="G36" s="386"/>
-      <c r="H36" s="386"/>
-      <c r="I36" s="386"/>
-      <c r="J36" s="386"/>
-      <c r="K36" s="386"/>
-      <c r="L36" s="386"/>
-      <c r="M36" s="386"/>
-      <c r="N36" s="386"/>
-      <c r="O36" s="386"/>
-      <c r="P36" s="386"/>
-      <c r="Q36" s="386"/>
-      <c r="R36" s="386"/>
+      <c r="B36" s="382"/>
+      <c r="C36" s="382"/>
+      <c r="D36" s="382"/>
+      <c r="E36" s="382"/>
+      <c r="F36" s="382"/>
+      <c r="G36" s="382"/>
+      <c r="H36" s="382"/>
+      <c r="I36" s="382"/>
+      <c r="J36" s="382"/>
+      <c r="K36" s="382"/>
+      <c r="L36" s="382"/>
+      <c r="M36" s="382"/>
+      <c r="N36" s="382"/>
+      <c r="O36" s="382"/>
+      <c r="P36" s="382"/>
+      <c r="Q36" s="382"/>
+      <c r="R36" s="382"/>
     </row>
     <row r="37" spans="1:21" ht="18.75" customHeight="1">
-      <c r="A37" s="388" t="s">
+      <c r="A37" s="384" t="s">
         <v>509</v>
       </c>
-      <c r="B37" s="386"/>
-      <c r="C37" s="386"/>
-      <c r="D37" s="386"/>
-      <c r="E37" s="386"/>
-      <c r="F37" s="386"/>
-      <c r="G37" s="386"/>
-      <c r="H37" s="386"/>
-      <c r="I37" s="386"/>
-      <c r="J37" s="386"/>
-      <c r="K37" s="386"/>
-      <c r="L37" s="386"/>
-      <c r="M37" s="386"/>
-      <c r="N37" s="386"/>
-      <c r="O37" s="386"/>
-      <c r="P37" s="386"/>
-      <c r="Q37" s="386"/>
-      <c r="R37" s="386"/>
+      <c r="B37" s="382"/>
+      <c r="C37" s="382"/>
+      <c r="D37" s="382"/>
+      <c r="E37" s="382"/>
+      <c r="F37" s="382"/>
+      <c r="G37" s="382"/>
+      <c r="H37" s="382"/>
+      <c r="I37" s="382"/>
+      <c r="J37" s="382"/>
+      <c r="K37" s="382"/>
+      <c r="L37" s="382"/>
+      <c r="M37" s="382"/>
+      <c r="N37" s="382"/>
+      <c r="O37" s="382"/>
+      <c r="P37" s="382"/>
+      <c r="Q37" s="382"/>
+      <c r="R37" s="382"/>
     </row>
     <row r="38" spans="1:21" ht="30.75" customHeight="1">
-      <c r="A38" s="388" t="s">
+      <c r="A38" s="384" t="s">
         <v>510</v>
       </c>
-      <c r="B38" s="386"/>
-      <c r="C38" s="386"/>
-      <c r="D38" s="386"/>
-      <c r="E38" s="386"/>
-      <c r="F38" s="386"/>
-      <c r="G38" s="386"/>
-      <c r="H38" s="386"/>
-      <c r="I38" s="386"/>
-      <c r="J38" s="386"/>
-      <c r="K38" s="386"/>
-      <c r="L38" s="386"/>
-      <c r="M38" s="386"/>
-      <c r="N38" s="386"/>
-      <c r="O38" s="386"/>
-      <c r="P38" s="386"/>
-      <c r="Q38" s="386"/>
-      <c r="R38" s="386"/>
+      <c r="B38" s="382"/>
+      <c r="C38" s="382"/>
+      <c r="D38" s="382"/>
+      <c r="E38" s="382"/>
+      <c r="F38" s="382"/>
+      <c r="G38" s="382"/>
+      <c r="H38" s="382"/>
+      <c r="I38" s="382"/>
+      <c r="J38" s="382"/>
+      <c r="K38" s="382"/>
+      <c r="L38" s="382"/>
+      <c r="M38" s="382"/>
+      <c r="N38" s="382"/>
+      <c r="O38" s="382"/>
+      <c r="P38" s="382"/>
+      <c r="Q38" s="382"/>
+      <c r="R38" s="382"/>
     </row>
     <row r="39" spans="1:21" ht="18.75" customHeight="1">
-      <c r="A39" s="388" t="s">
+      <c r="A39" s="384" t="s">
         <v>511</v>
       </c>
-      <c r="B39" s="386"/>
-      <c r="C39" s="386"/>
-      <c r="D39" s="386"/>
-      <c r="E39" s="386"/>
-      <c r="F39" s="386"/>
-      <c r="G39" s="386"/>
-      <c r="H39" s="386"/>
-      <c r="I39" s="386"/>
-      <c r="J39" s="386"/>
-      <c r="K39" s="386"/>
-      <c r="L39" s="386"/>
-      <c r="M39" s="386"/>
-      <c r="N39" s="386"/>
-      <c r="O39" s="386"/>
-      <c r="P39" s="386"/>
-      <c r="Q39" s="386"/>
-      <c r="R39" s="386"/>
+      <c r="B39" s="382"/>
+      <c r="C39" s="382"/>
+      <c r="D39" s="382"/>
+      <c r="E39" s="382"/>
+      <c r="F39" s="382"/>
+      <c r="G39" s="382"/>
+      <c r="H39" s="382"/>
+      <c r="I39" s="382"/>
+      <c r="J39" s="382"/>
+      <c r="K39" s="382"/>
+      <c r="L39" s="382"/>
+      <c r="M39" s="382"/>
+      <c r="N39" s="382"/>
+      <c r="O39" s="382"/>
+      <c r="P39" s="382"/>
+      <c r="Q39" s="382"/>
+      <c r="R39" s="382"/>
     </row>
     <row r="40" spans="1:21" ht="17.25" customHeight="1">
-      <c r="A40" s="384" t="s">
+      <c r="A40" s="380" t="s">
         <v>661</v>
       </c>
-      <c r="B40" s="384"/>
-      <c r="C40" s="384"/>
-      <c r="D40" s="384"/>
-      <c r="E40" s="384"/>
-      <c r="F40" s="384"/>
-      <c r="G40" s="384"/>
-      <c r="H40" s="384"/>
-      <c r="I40" s="384"/>
-      <c r="J40" s="384"/>
-      <c r="K40" s="384"/>
-      <c r="L40" s="384"/>
-      <c r="M40" s="384"/>
-      <c r="N40" s="384"/>
-      <c r="O40" s="384"/>
-      <c r="P40" s="384"/>
-      <c r="Q40" s="384"/>
-      <c r="R40" s="384"/>
+      <c r="B40" s="380"/>
+      <c r="C40" s="380"/>
+      <c r="D40" s="380"/>
+      <c r="E40" s="380"/>
+      <c r="F40" s="380"/>
+      <c r="G40" s="380"/>
+      <c r="H40" s="380"/>
+      <c r="I40" s="380"/>
+      <c r="J40" s="380"/>
+      <c r="K40" s="380"/>
+      <c r="L40" s="380"/>
+      <c r="M40" s="380"/>
+      <c r="N40" s="380"/>
+      <c r="O40" s="380"/>
+      <c r="P40" s="380"/>
+      <c r="Q40" s="380"/>
+      <c r="R40" s="380"/>
       <c r="S40" s="168"/>
       <c r="T40" s="168"/>
       <c r="U40" s="168"/>
     </row>
     <row r="41" spans="1:21" ht="17.25" customHeight="1">
-      <c r="A41" s="384"/>
-      <c r="B41" s="384"/>
-      <c r="C41" s="384"/>
-      <c r="D41" s="384"/>
-      <c r="E41" s="384"/>
-      <c r="F41" s="384"/>
-      <c r="G41" s="384"/>
-      <c r="H41" s="384"/>
-      <c r="I41" s="384"/>
-      <c r="J41" s="384"/>
-      <c r="K41" s="384"/>
-      <c r="L41" s="384"/>
-      <c r="M41" s="384"/>
-      <c r="N41" s="384"/>
-      <c r="O41" s="384"/>
-      <c r="P41" s="384"/>
-      <c r="Q41" s="384"/>
-      <c r="R41" s="384"/>
+      <c r="A41" s="380"/>
+      <c r="B41" s="380"/>
+      <c r="C41" s="380"/>
+      <c r="D41" s="380"/>
+      <c r="E41" s="380"/>
+      <c r="F41" s="380"/>
+      <c r="G41" s="380"/>
+      <c r="H41" s="380"/>
+      <c r="I41" s="380"/>
+      <c r="J41" s="380"/>
+      <c r="K41" s="380"/>
+      <c r="L41" s="380"/>
+      <c r="M41" s="380"/>
+      <c r="N41" s="380"/>
+      <c r="O41" s="380"/>
+      <c r="P41" s="380"/>
+      <c r="Q41" s="380"/>
+      <c r="R41" s="380"/>
       <c r="S41" s="168"/>
       <c r="T41" s="168"/>
       <c r="U41" s="168"/>
     </row>
     <row r="42" spans="1:21" ht="18.75" customHeight="1">
-      <c r="A42" s="384" t="s">
+      <c r="A42" s="380" t="s">
         <v>659</v>
       </c>
-      <c r="B42" s="384"/>
-      <c r="C42" s="384"/>
-      <c r="D42" s="384"/>
-      <c r="E42" s="384"/>
-      <c r="F42" s="384"/>
-      <c r="G42" s="384"/>
-      <c r="H42" s="384"/>
-      <c r="I42" s="384"/>
-      <c r="J42" s="384"/>
-      <c r="K42" s="384"/>
-      <c r="L42" s="384"/>
-      <c r="M42" s="384"/>
-      <c r="N42" s="384"/>
-      <c r="O42" s="384"/>
-      <c r="P42" s="384"/>
-      <c r="Q42" s="384"/>
-      <c r="R42" s="384"/>
+      <c r="B42" s="380"/>
+      <c r="C42" s="380"/>
+      <c r="D42" s="380"/>
+      <c r="E42" s="380"/>
+      <c r="F42" s="380"/>
+      <c r="G42" s="380"/>
+      <c r="H42" s="380"/>
+      <c r="I42" s="380"/>
+      <c r="J42" s="380"/>
+      <c r="K42" s="380"/>
+      <c r="L42" s="380"/>
+      <c r="M42" s="380"/>
+      <c r="N42" s="380"/>
+      <c r="O42" s="380"/>
+      <c r="P42" s="380"/>
+      <c r="Q42" s="380"/>
+      <c r="R42" s="380"/>
       <c r="S42" s="168"/>
       <c r="T42" s="168"/>
       <c r="U42" s="168"/>
@@ -45296,22 +45273,22 @@
       <c r="M46" s="39"/>
     </row>
     <row r="47" spans="1:14" ht="51.75" customHeight="1">
-      <c r="A47" s="368" t="s">
+      <c r="A47" s="386" t="s">
         <v>737</v>
       </c>
-      <c r="B47" s="368"/>
-      <c r="C47" s="368"/>
-      <c r="D47" s="368"/>
-      <c r="E47" s="368"/>
-      <c r="F47" s="368"/>
-      <c r="G47" s="368"/>
-      <c r="H47" s="368"/>
-      <c r="I47" s="368"/>
-      <c r="J47" s="368"/>
-      <c r="K47" s="368"/>
-      <c r="L47" s="368"/>
-      <c r="M47" s="368"/>
-      <c r="N47" s="368"/>
+      <c r="B47" s="386"/>
+      <c r="C47" s="386"/>
+      <c r="D47" s="386"/>
+      <c r="E47" s="386"/>
+      <c r="F47" s="386"/>
+      <c r="G47" s="386"/>
+      <c r="H47" s="386"/>
+      <c r="I47" s="386"/>
+      <c r="J47" s="386"/>
+      <c r="K47" s="386"/>
+      <c r="L47" s="386"/>
+      <c r="M47" s="386"/>
+      <c r="N47" s="386"/>
     </row>
     <row r="48" spans="1:14">
       <c r="C48" s="29"/>
@@ -45327,190 +45304,190 @@
       <c r="M48" s="29"/>
     </row>
     <row r="49" spans="1:18" customFormat="1" ht="30.75" customHeight="1">
-      <c r="A49" s="391" t="s">
+      <c r="A49" s="388" t="s">
         <v>514</v>
       </c>
-      <c r="B49" s="391"/>
-      <c r="C49" s="391"/>
-      <c r="D49" s="391"/>
-      <c r="E49" s="391"/>
-      <c r="F49" s="391"/>
-      <c r="G49" s="391"/>
-      <c r="H49" s="391"/>
-      <c r="I49" s="391"/>
-      <c r="J49" s="391"/>
-      <c r="K49" s="391"/>
-      <c r="L49" s="391"/>
-      <c r="M49" s="391"/>
-      <c r="N49" s="391"/>
+      <c r="B49" s="388"/>
+      <c r="C49" s="388"/>
+      <c r="D49" s="388"/>
+      <c r="E49" s="388"/>
+      <c r="F49" s="388"/>
+      <c r="G49" s="388"/>
+      <c r="H49" s="388"/>
+      <c r="I49" s="388"/>
+      <c r="J49" s="388"/>
+      <c r="K49" s="388"/>
+      <c r="L49" s="388"/>
+      <c r="M49" s="388"/>
+      <c r="N49" s="388"/>
       <c r="O49" s="44"/>
       <c r="P49" s="44"/>
       <c r="Q49" s="44"/>
       <c r="R49" s="44"/>
     </row>
     <row r="50" spans="1:18" customFormat="1" ht="17.25" customHeight="1">
-      <c r="A50" s="391" t="s">
+      <c r="A50" s="388" t="s">
         <v>117</v>
       </c>
-      <c r="B50" s="394"/>
-      <c r="C50" s="394"/>
-      <c r="D50" s="394"/>
-      <c r="E50" s="394"/>
-      <c r="F50" s="394"/>
-      <c r="G50" s="394"/>
-      <c r="H50" s="394"/>
-      <c r="I50" s="394"/>
-      <c r="J50" s="394"/>
-      <c r="K50" s="394"/>
-      <c r="L50" s="394"/>
-      <c r="M50" s="394"/>
-      <c r="N50" s="394"/>
+      <c r="B50" s="391"/>
+      <c r="C50" s="391"/>
+      <c r="D50" s="391"/>
+      <c r="E50" s="391"/>
+      <c r="F50" s="391"/>
+      <c r="G50" s="391"/>
+      <c r="H50" s="391"/>
+      <c r="I50" s="391"/>
+      <c r="J50" s="391"/>
+      <c r="K50" s="391"/>
+      <c r="L50" s="391"/>
+      <c r="M50" s="391"/>
+      <c r="N50" s="391"/>
       <c r="O50" s="44"/>
       <c r="P50" s="44"/>
       <c r="Q50" s="44"/>
       <c r="R50" s="44"/>
     </row>
     <row r="51" spans="1:18" customFormat="1" ht="32.25" customHeight="1">
-      <c r="A51" s="391" t="s">
+      <c r="A51" s="388" t="s">
         <v>54</v>
       </c>
-      <c r="B51" s="394"/>
-      <c r="C51" s="394"/>
-      <c r="D51" s="394"/>
-      <c r="E51" s="394"/>
-      <c r="F51" s="394"/>
-      <c r="G51" s="394"/>
-      <c r="H51" s="394"/>
-      <c r="I51" s="394"/>
-      <c r="J51" s="394"/>
-      <c r="K51" s="394"/>
-      <c r="L51" s="394"/>
-      <c r="M51" s="394"/>
-      <c r="N51" s="394"/>
+      <c r="B51" s="391"/>
+      <c r="C51" s="391"/>
+      <c r="D51" s="391"/>
+      <c r="E51" s="391"/>
+      <c r="F51" s="391"/>
+      <c r="G51" s="391"/>
+      <c r="H51" s="391"/>
+      <c r="I51" s="391"/>
+      <c r="J51" s="391"/>
+      <c r="K51" s="391"/>
+      <c r="L51" s="391"/>
+      <c r="M51" s="391"/>
+      <c r="N51" s="391"/>
       <c r="O51" s="44"/>
       <c r="P51" s="44"/>
       <c r="Q51" s="44"/>
       <c r="R51" s="44"/>
     </row>
     <row r="52" spans="1:18" customFormat="1" ht="30.75" customHeight="1">
-      <c r="A52" s="391" t="s">
+      <c r="A52" s="388" t="s">
         <v>55</v>
       </c>
-      <c r="B52" s="393"/>
-      <c r="C52" s="393"/>
-      <c r="D52" s="393"/>
-      <c r="E52" s="393"/>
-      <c r="F52" s="393"/>
-      <c r="G52" s="393"/>
-      <c r="H52" s="393"/>
-      <c r="I52" s="393"/>
-      <c r="J52" s="393"/>
-      <c r="K52" s="393"/>
-      <c r="L52" s="393"/>
-      <c r="M52" s="393"/>
-      <c r="N52" s="393"/>
+      <c r="B52" s="390"/>
+      <c r="C52" s="390"/>
+      <c r="D52" s="390"/>
+      <c r="E52" s="390"/>
+      <c r="F52" s="390"/>
+      <c r="G52" s="390"/>
+      <c r="H52" s="390"/>
+      <c r="I52" s="390"/>
+      <c r="J52" s="390"/>
+      <c r="K52" s="390"/>
+      <c r="L52" s="390"/>
+      <c r="M52" s="390"/>
+      <c r="N52" s="390"/>
       <c r="O52" s="44"/>
       <c r="P52" s="44"/>
       <c r="Q52" s="44"/>
       <c r="R52" s="44"/>
     </row>
     <row r="53" spans="1:18" customFormat="1" ht="46.5" customHeight="1">
-      <c r="A53" s="392" t="s">
+      <c r="A53" s="389" t="s">
         <v>642</v>
       </c>
-      <c r="B53" s="392"/>
-      <c r="C53" s="392"/>
-      <c r="D53" s="392"/>
-      <c r="E53" s="392"/>
-      <c r="F53" s="392"/>
-      <c r="G53" s="392"/>
-      <c r="H53" s="392"/>
-      <c r="I53" s="392"/>
-      <c r="J53" s="392"/>
-      <c r="K53" s="392"/>
-      <c r="L53" s="392"/>
-      <c r="M53" s="392"/>
-      <c r="N53" s="392"/>
+      <c r="B53" s="389"/>
+      <c r="C53" s="389"/>
+      <c r="D53" s="389"/>
+      <c r="E53" s="389"/>
+      <c r="F53" s="389"/>
+      <c r="G53" s="389"/>
+      <c r="H53" s="389"/>
+      <c r="I53" s="389"/>
+      <c r="J53" s="389"/>
+      <c r="K53" s="389"/>
+      <c r="L53" s="389"/>
+      <c r="M53" s="389"/>
+      <c r="N53" s="389"/>
       <c r="O53" s="170"/>
       <c r="P53" s="170"/>
       <c r="Q53" s="170"/>
       <c r="R53" s="170"/>
     </row>
     <row r="54" spans="1:18" customFormat="1" ht="17.25" customHeight="1">
-      <c r="A54" s="390" t="s">
+      <c r="A54" s="387" t="s">
         <v>643</v>
       </c>
-      <c r="B54" s="390"/>
-      <c r="C54" s="390"/>
-      <c r="D54" s="390"/>
-      <c r="E54" s="390"/>
-      <c r="F54" s="390"/>
-      <c r="G54" s="390"/>
-      <c r="H54" s="390"/>
-      <c r="I54" s="390"/>
-      <c r="J54" s="390"/>
-      <c r="K54" s="390"/>
-      <c r="L54" s="390"/>
-      <c r="M54" s="390"/>
-      <c r="N54" s="390"/>
+      <c r="B54" s="387"/>
+      <c r="C54" s="387"/>
+      <c r="D54" s="387"/>
+      <c r="E54" s="387"/>
+      <c r="F54" s="387"/>
+      <c r="G54" s="387"/>
+      <c r="H54" s="387"/>
+      <c r="I54" s="387"/>
+      <c r="J54" s="387"/>
+      <c r="K54" s="387"/>
+      <c r="L54" s="387"/>
+      <c r="M54" s="387"/>
+      <c r="N54" s="387"/>
       <c r="O54" s="44"/>
       <c r="P54" s="44"/>
       <c r="Q54" s="44"/>
       <c r="R54" s="44"/>
     </row>
     <row r="55" spans="1:18" customFormat="1" ht="30.75" customHeight="1">
-      <c r="A55" s="392" t="s">
+      <c r="A55" s="389" t="s">
         <v>674</v>
       </c>
-      <c r="B55" s="393"/>
-      <c r="C55" s="393"/>
-      <c r="D55" s="393"/>
-      <c r="E55" s="393"/>
-      <c r="F55" s="393"/>
-      <c r="G55" s="393"/>
-      <c r="H55" s="393"/>
-      <c r="I55" s="393"/>
-      <c r="J55" s="393"/>
-      <c r="K55" s="393"/>
-      <c r="L55" s="393"/>
-      <c r="M55" s="393"/>
-      <c r="N55" s="393"/>
+      <c r="B55" s="390"/>
+      <c r="C55" s="390"/>
+      <c r="D55" s="390"/>
+      <c r="E55" s="390"/>
+      <c r="F55" s="390"/>
+      <c r="G55" s="390"/>
+      <c r="H55" s="390"/>
+      <c r="I55" s="390"/>
+      <c r="J55" s="390"/>
+      <c r="K55" s="390"/>
+      <c r="L55" s="390"/>
+      <c r="M55" s="390"/>
+      <c r="N55" s="390"/>
       <c r="O55" s="44"/>
       <c r="P55" s="44"/>
       <c r="Q55" s="44"/>
       <c r="R55" s="44"/>
     </row>
     <row r="56" spans="1:18" customFormat="1" ht="17.25" customHeight="1">
-      <c r="A56" s="392" t="s">
+      <c r="A56" s="389" t="s">
         <v>644</v>
       </c>
-      <c r="B56" s="393"/>
-      <c r="C56" s="393"/>
-      <c r="D56" s="393"/>
-      <c r="E56" s="393"/>
-      <c r="F56" s="393"/>
-      <c r="G56" s="393"/>
-      <c r="H56" s="393"/>
-      <c r="I56" s="393"/>
-      <c r="J56" s="393"/>
-      <c r="K56" s="393"/>
-      <c r="L56" s="393"/>
-      <c r="M56" s="393"/>
-      <c r="N56" s="393"/>
+      <c r="B56" s="390"/>
+      <c r="C56" s="390"/>
+      <c r="D56" s="390"/>
+      <c r="E56" s="390"/>
+      <c r="F56" s="390"/>
+      <c r="G56" s="390"/>
+      <c r="H56" s="390"/>
+      <c r="I56" s="390"/>
+      <c r="J56" s="390"/>
+      <c r="K56" s="390"/>
+      <c r="L56" s="390"/>
+      <c r="M56" s="390"/>
+      <c r="N56" s="390"/>
       <c r="O56" s="44"/>
       <c r="P56" s="44"/>
       <c r="Q56" s="44"/>
       <c r="R56" s="44"/>
     </row>
     <row r="57" spans="1:18" customFormat="1" ht="17.25" customHeight="1">
-      <c r="A57" s="390" t="s">
+      <c r="A57" s="387" t="s">
         <v>645</v>
       </c>
-      <c r="B57" s="390"/>
-      <c r="C57" s="390"/>
-      <c r="D57" s="390"/>
-      <c r="E57" s="390"/>
-      <c r="F57" s="390"/>
+      <c r="B57" s="387"/>
+      <c r="C57" s="387"/>
+      <c r="D57" s="387"/>
+      <c r="E57" s="387"/>
+      <c r="F57" s="387"/>
       <c r="G57" s="355"/>
       <c r="H57" s="355"/>
       <c r="I57" s="355"/>
@@ -45525,22 +45502,22 @@
       <c r="R57" s="44"/>
     </row>
     <row r="58" spans="1:18" customFormat="1" ht="17.25" customHeight="1">
-      <c r="A58" s="389" t="s">
+      <c r="A58" s="385" t="s">
         <v>662</v>
       </c>
-      <c r="B58" s="389"/>
-      <c r="C58" s="389"/>
-      <c r="D58" s="389"/>
-      <c r="E58" s="389"/>
-      <c r="F58" s="389"/>
-      <c r="G58" s="389"/>
-      <c r="H58" s="389"/>
-      <c r="I58" s="389"/>
-      <c r="J58" s="389"/>
-      <c r="K58" s="389"/>
-      <c r="L58" s="389"/>
-      <c r="M58" s="389"/>
-      <c r="N58" s="389"/>
+      <c r="B58" s="385"/>
+      <c r="C58" s="385"/>
+      <c r="D58" s="385"/>
+      <c r="E58" s="385"/>
+      <c r="F58" s="385"/>
+      <c r="G58" s="385"/>
+      <c r="H58" s="385"/>
+      <c r="I58" s="385"/>
+      <c r="J58" s="385"/>
+      <c r="K58" s="385"/>
+      <c r="L58" s="385"/>
+      <c r="M58" s="385"/>
+      <c r="N58" s="385"/>
       <c r="O58" s="44"/>
       <c r="P58" s="44"/>
       <c r="Q58" s="44"/>
@@ -46622,10 +46599,10 @@
       <c r="A5" s="59"/>
       <c r="B5" s="132"/>
       <c r="C5" s="60"/>
-      <c r="D5" s="395" t="s">
+      <c r="D5" s="392" t="s">
         <v>548</v>
       </c>
-      <c r="E5" s="395"/>
+      <c r="E5" s="392"/>
       <c r="F5"/>
       <c r="G5" s="60"/>
       <c r="H5" s="60"/>
@@ -46852,10 +46829,10 @@
       <c r="A6" s="59"/>
       <c r="B6" s="132"/>
       <c r="C6" s="60"/>
-      <c r="D6" s="395" t="s">
+      <c r="D6" s="392" t="s">
         <v>549</v>
       </c>
-      <c r="E6" s="395"/>
+      <c r="E6" s="392"/>
       <c r="F6"/>
       <c r="G6" s="60"/>
       <c r="H6" s="60"/>
@@ -63588,21 +63565,21 @@
       <c r="E2" s="167"/>
     </row>
     <row r="3" spans="1:13" ht="44.25" customHeight="1">
-      <c r="A3" s="396" t="s">
+      <c r="A3" s="393" t="s">
         <v>646</v>
       </c>
-      <c r="B3" s="396"/>
-      <c r="C3" s="396"/>
-      <c r="D3" s="396"/>
-      <c r="E3" s="396"/>
-      <c r="F3" s="396"/>
-      <c r="G3" s="396"/>
-      <c r="H3" s="396"/>
-      <c r="I3" s="396"/>
-      <c r="J3" s="396"/>
-      <c r="K3" s="396"/>
-      <c r="L3" s="396"/>
-      <c r="M3" s="396"/>
+      <c r="B3" s="393"/>
+      <c r="C3" s="393"/>
+      <c r="D3" s="393"/>
+      <c r="E3" s="393"/>
+      <c r="F3" s="393"/>
+      <c r="G3" s="393"/>
+      <c r="H3" s="393"/>
+      <c r="I3" s="393"/>
+      <c r="J3" s="393"/>
+      <c r="K3" s="393"/>
+      <c r="L3" s="393"/>
+      <c r="M3" s="393"/>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="263"/>
@@ -63650,21 +63627,21 @@
       <c r="M9" s="22"/>
     </row>
     <row r="10" spans="1:13" ht="48.75" customHeight="1">
-      <c r="A10" s="397" t="s">
+      <c r="A10" s="394" t="s">
         <v>588</v>
       </c>
-      <c r="B10" s="397"/>
-      <c r="C10" s="397"/>
-      <c r="D10" s="397"/>
-      <c r="E10" s="397"/>
-      <c r="F10" s="397"/>
-      <c r="G10" s="397"/>
-      <c r="H10" s="397"/>
-      <c r="I10" s="397"/>
-      <c r="J10" s="397"/>
-      <c r="K10" s="397"/>
-      <c r="L10" s="397"/>
-      <c r="M10" s="397"/>
+      <c r="B10" s="394"/>
+      <c r="C10" s="394"/>
+      <c r="D10" s="394"/>
+      <c r="E10" s="394"/>
+      <c r="F10" s="394"/>
+      <c r="G10" s="394"/>
+      <c r="H10" s="394"/>
+      <c r="I10" s="394"/>
+      <c r="J10" s="394"/>
+      <c r="K10" s="394"/>
+      <c r="L10" s="394"/>
+      <c r="M10" s="394"/>
     </row>
     <row r="11" spans="1:13">
       <c r="A11" s="264"/>
@@ -64276,55 +64253,55 @@
       <c r="M39" s="22"/>
     </row>
     <row r="40" spans="1:13" ht="48" customHeight="1">
-      <c r="A40" s="398" t="s">
+      <c r="A40" s="395" t="s">
         <v>584</v>
       </c>
-      <c r="B40" s="386"/>
-      <c r="C40" s="386"/>
-      <c r="D40" s="386"/>
-      <c r="E40" s="386"/>
-      <c r="F40" s="386"/>
-      <c r="G40" s="386"/>
-      <c r="H40" s="386"/>
-      <c r="I40" s="386"/>
-      <c r="J40" s="386"/>
-      <c r="K40" s="386"/>
-      <c r="L40" s="386"/>
-      <c r="M40" s="386"/>
+      <c r="B40" s="382"/>
+      <c r="C40" s="382"/>
+      <c r="D40" s="382"/>
+      <c r="E40" s="382"/>
+      <c r="F40" s="382"/>
+      <c r="G40" s="382"/>
+      <c r="H40" s="382"/>
+      <c r="I40" s="382"/>
+      <c r="J40" s="382"/>
+      <c r="K40" s="382"/>
+      <c r="L40" s="382"/>
+      <c r="M40" s="382"/>
     </row>
     <row r="41" spans="1:13" ht="50.25" customHeight="1">
-      <c r="A41" s="399" t="s">
+      <c r="A41" s="396" t="s">
         <v>668</v>
       </c>
-      <c r="B41" s="400"/>
-      <c r="C41" s="400"/>
-      <c r="D41" s="400"/>
-      <c r="E41" s="400"/>
-      <c r="F41" s="400"/>
-      <c r="G41" s="400"/>
-      <c r="H41" s="400"/>
-      <c r="I41" s="400"/>
-      <c r="J41" s="400"/>
-      <c r="K41" s="400"/>
-      <c r="L41" s="400"/>
-      <c r="M41" s="400"/>
+      <c r="B41" s="397"/>
+      <c r="C41" s="397"/>
+      <c r="D41" s="397"/>
+      <c r="E41" s="397"/>
+      <c r="F41" s="397"/>
+      <c r="G41" s="397"/>
+      <c r="H41" s="397"/>
+      <c r="I41" s="397"/>
+      <c r="J41" s="397"/>
+      <c r="K41" s="397"/>
+      <c r="L41" s="397"/>
+      <c r="M41" s="397"/>
     </row>
     <row r="42" spans="1:13" ht="21" customHeight="1">
-      <c r="A42" s="401" t="s">
+      <c r="A42" s="398" t="s">
         <v>647</v>
       </c>
-      <c r="B42" s="401"/>
-      <c r="C42" s="401"/>
-      <c r="D42" s="401"/>
-      <c r="E42" s="401"/>
-      <c r="F42" s="401"/>
-      <c r="G42" s="401"/>
-      <c r="H42" s="401"/>
-      <c r="I42" s="401"/>
-      <c r="J42" s="401"/>
-      <c r="K42" s="401"/>
-      <c r="L42" s="401"/>
-      <c r="M42" s="401"/>
+      <c r="B42" s="398"/>
+      <c r="C42" s="398"/>
+      <c r="D42" s="398"/>
+      <c r="E42" s="398"/>
+      <c r="F42" s="398"/>
+      <c r="G42" s="398"/>
+      <c r="H42" s="398"/>
+      <c r="I42" s="398"/>
+      <c r="J42" s="398"/>
+      <c r="K42" s="398"/>
+      <c r="L42" s="398"/>
+      <c r="M42" s="398"/>
     </row>
     <row r="43" spans="1:13" ht="15.75">
       <c r="B43" s="22"/>
@@ -64389,17 +64366,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="84.95" customHeight="1">
-      <c r="A1" s="403" t="s">
+      <c r="A1" s="402" t="s">
         <v>738</v>
       </c>
-      <c r="B1" s="403"/>
-      <c r="C1" s="403"/>
+      <c r="B1" s="402"/>
+      <c r="C1" s="402"/>
       <c r="D1" s="281"/>
-      <c r="E1" s="403" t="s">
+      <c r="E1" s="402" t="s">
         <v>739</v>
       </c>
-      <c r="F1" s="403"/>
-      <c r="G1" s="403"/>
+      <c r="F1" s="402"/>
+      <c r="G1" s="402"/>
     </row>
     <row r="2" spans="1:7" ht="9" customHeight="1">
       <c r="A2" s="1"/>
@@ -64834,16 +64811,16 @@
       <c r="F35" s="1"/>
     </row>
     <row r="36" spans="1:16" s="302" customFormat="1" ht="14.25" customHeight="1">
-      <c r="A36" s="404" t="s">
+      <c r="A36" s="403" t="s">
         <v>66</v>
       </c>
-      <c r="B36" s="404"/>
-      <c r="C36" s="404"/>
-      <c r="D36" s="404"/>
-      <c r="E36" s="404"/>
-      <c r="F36" s="404"/>
-      <c r="G36" s="404"/>
-      <c r="H36" s="404"/>
+      <c r="B36" s="403"/>
+      <c r="C36" s="403"/>
+      <c r="D36" s="403"/>
+      <c r="E36" s="403"/>
+      <c r="F36" s="403"/>
+      <c r="G36" s="403"/>
+      <c r="H36" s="403"/>
       <c r="I36" s="44"/>
       <c r="J36" s="44"/>
       <c r="K36" s="44"/>
@@ -64872,16 +64849,16 @@
       <c r="P37" s="44"/>
     </row>
     <row r="38" spans="1:16" s="302" customFormat="1" ht="33.75" customHeight="1">
-      <c r="A38" s="405" t="s">
+      <c r="A38" s="400" t="s">
         <v>613</v>
       </c>
-      <c r="B38" s="405"/>
-      <c r="C38" s="405"/>
-      <c r="D38" s="405"/>
-      <c r="E38" s="405"/>
-      <c r="F38" s="405"/>
-      <c r="G38" s="405"/>
-      <c r="H38" s="405"/>
+      <c r="B38" s="400"/>
+      <c r="C38" s="400"/>
+      <c r="D38" s="400"/>
+      <c r="E38" s="400"/>
+      <c r="F38" s="400"/>
+      <c r="G38" s="400"/>
+      <c r="H38" s="400"/>
       <c r="I38" s="290"/>
       <c r="J38" s="44"/>
       <c r="K38" s="44"/>
@@ -64892,16 +64869,16 @@
       <c r="P38" s="44"/>
     </row>
     <row r="39" spans="1:16" s="302" customFormat="1" ht="33.75" customHeight="1">
-      <c r="A39" s="405" t="s">
+      <c r="A39" s="400" t="s">
         <v>673</v>
       </c>
-      <c r="B39" s="405"/>
-      <c r="C39" s="405"/>
-      <c r="D39" s="405"/>
-      <c r="E39" s="405"/>
-      <c r="F39" s="405"/>
-      <c r="G39" s="405"/>
-      <c r="H39" s="405"/>
+      <c r="B39" s="400"/>
+      <c r="C39" s="400"/>
+      <c r="D39" s="400"/>
+      <c r="E39" s="400"/>
+      <c r="F39" s="400"/>
+      <c r="G39" s="400"/>
+      <c r="H39" s="400"/>
       <c r="I39" s="290"/>
       <c r="J39" s="44"/>
       <c r="K39" s="44"/>
@@ -64912,16 +64889,16 @@
       <c r="P39" s="44"/>
     </row>
     <row r="40" spans="1:16" s="302" customFormat="1" ht="33.75" customHeight="1">
-      <c r="A40" s="405" t="s">
+      <c r="A40" s="400" t="s">
         <v>614</v>
       </c>
-      <c r="B40" s="405"/>
-      <c r="C40" s="405"/>
-      <c r="D40" s="405"/>
-      <c r="E40" s="405"/>
-      <c r="F40" s="405"/>
-      <c r="G40" s="405"/>
-      <c r="H40" s="405"/>
+      <c r="B40" s="400"/>
+      <c r="C40" s="400"/>
+      <c r="D40" s="400"/>
+      <c r="E40" s="400"/>
+      <c r="F40" s="400"/>
+      <c r="G40" s="400"/>
+      <c r="H40" s="400"/>
       <c r="I40" s="290"/>
       <c r="J40" s="44"/>
       <c r="K40" s="44"/>
@@ -64932,16 +64909,16 @@
       <c r="P40" s="44"/>
     </row>
     <row r="41" spans="1:16" s="302" customFormat="1" ht="33.75" customHeight="1">
-      <c r="A41" s="405" t="s">
+      <c r="A41" s="400" t="s">
         <v>669</v>
       </c>
-      <c r="B41" s="405"/>
-      <c r="C41" s="405"/>
-      <c r="D41" s="405"/>
-      <c r="E41" s="405"/>
-      <c r="F41" s="405"/>
-      <c r="G41" s="405"/>
-      <c r="H41" s="405"/>
+      <c r="B41" s="400"/>
+      <c r="C41" s="400"/>
+      <c r="D41" s="400"/>
+      <c r="E41" s="400"/>
+      <c r="F41" s="400"/>
+      <c r="G41" s="400"/>
+      <c r="H41" s="400"/>
       <c r="I41" s="290"/>
       <c r="J41" s="44"/>
       <c r="K41" s="44"/>
@@ -64952,16 +64929,16 @@
       <c r="P41" s="44"/>
     </row>
     <row r="42" spans="1:16" s="302" customFormat="1" ht="65.099999999999994" customHeight="1">
-      <c r="A42" s="405" t="s">
+      <c r="A42" s="400" t="s">
         <v>615</v>
       </c>
-      <c r="B42" s="405"/>
-      <c r="C42" s="405"/>
-      <c r="D42" s="405"/>
-      <c r="E42" s="405"/>
-      <c r="F42" s="405"/>
-      <c r="G42" s="405"/>
-      <c r="H42" s="405"/>
+      <c r="B42" s="400"/>
+      <c r="C42" s="400"/>
+      <c r="D42" s="400"/>
+      <c r="E42" s="400"/>
+      <c r="F42" s="400"/>
+      <c r="G42" s="400"/>
+      <c r="H42" s="400"/>
       <c r="I42" s="291"/>
       <c r="J42" s="22"/>
       <c r="K42" s="22"/>
@@ -64972,16 +64949,16 @@
       <c r="P42" s="22"/>
     </row>
     <row r="43" spans="1:16" s="302" customFormat="1" ht="20.100000000000001" customHeight="1">
-      <c r="A43" s="405" t="s">
+      <c r="A43" s="400" t="s">
         <v>616</v>
       </c>
-      <c r="B43" s="405"/>
-      <c r="C43" s="405"/>
-      <c r="D43" s="405"/>
-      <c r="E43" s="405"/>
-      <c r="F43" s="405"/>
-      <c r="G43" s="405"/>
-      <c r="H43" s="405"/>
+      <c r="B43" s="400"/>
+      <c r="C43" s="400"/>
+      <c r="D43" s="400"/>
+      <c r="E43" s="400"/>
+      <c r="F43" s="400"/>
+      <c r="G43" s="400"/>
+      <c r="H43" s="400"/>
       <c r="I43" s="290"/>
       <c r="J43" s="44"/>
       <c r="K43" s="44"/>
@@ -64992,56 +64969,56 @@
       <c r="P43" s="44"/>
     </row>
     <row r="44" spans="1:16" s="302" customFormat="1" ht="50.1" customHeight="1">
-      <c r="A44" s="405" t="s">
+      <c r="A44" s="400" t="s">
         <v>672</v>
       </c>
-      <c r="B44" s="405"/>
-      <c r="C44" s="405"/>
-      <c r="D44" s="405"/>
-      <c r="E44" s="405"/>
-      <c r="F44" s="405"/>
-      <c r="G44" s="405"/>
-      <c r="H44" s="405"/>
+      <c r="B44" s="400"/>
+      <c r="C44" s="400"/>
+      <c r="D44" s="400"/>
+      <c r="E44" s="400"/>
+      <c r="F44" s="400"/>
+      <c r="G44" s="400"/>
+      <c r="H44" s="400"/>
       <c r="I44" s="290"/>
       <c r="J44" s="44"/>
       <c r="K44" s="44"/>
       <c r="L44" s="44"/>
-      <c r="M44" s="381"/>
-      <c r="N44" s="367"/>
-      <c r="O44" s="367"/>
-      <c r="P44" s="367"/>
+      <c r="M44" s="377"/>
+      <c r="N44" s="399"/>
+      <c r="O44" s="399"/>
+      <c r="P44" s="399"/>
     </row>
     <row r="45" spans="1:16" s="302" customFormat="1" ht="20.100000000000001" customHeight="1">
-      <c r="A45" s="405" t="s">
+      <c r="A45" s="400" t="s">
         <v>617</v>
       </c>
-      <c r="B45" s="405"/>
-      <c r="C45" s="405"/>
-      <c r="D45" s="405"/>
-      <c r="E45" s="405"/>
-      <c r="F45" s="405"/>
-      <c r="G45" s="405"/>
-      <c r="H45" s="405"/>
+      <c r="B45" s="400"/>
+      <c r="C45" s="400"/>
+      <c r="D45" s="400"/>
+      <c r="E45" s="400"/>
+      <c r="F45" s="400"/>
+      <c r="G45" s="400"/>
+      <c r="H45" s="400"/>
       <c r="I45" s="290"/>
       <c r="J45" s="44"/>
       <c r="K45" s="44"/>
       <c r="L45" s="44"/>
-      <c r="M45" s="381"/>
-      <c r="N45" s="367"/>
-      <c r="O45" s="367"/>
-      <c r="P45" s="367"/>
+      <c r="M45" s="377"/>
+      <c r="N45" s="399"/>
+      <c r="O45" s="399"/>
+      <c r="P45" s="399"/>
     </row>
     <row r="46" spans="1:16" ht="20.100000000000001" customHeight="1">
-      <c r="A46" s="405" t="s">
+      <c r="A46" s="400" t="s">
         <v>618</v>
       </c>
-      <c r="B46" s="405"/>
-      <c r="C46" s="405"/>
-      <c r="D46" s="405"/>
-      <c r="E46" s="405"/>
-      <c r="F46" s="405"/>
-      <c r="G46" s="405"/>
-      <c r="H46" s="405"/>
+      <c r="B46" s="400"/>
+      <c r="C46" s="400"/>
+      <c r="D46" s="400"/>
+      <c r="E46" s="400"/>
+      <c r="F46" s="400"/>
+      <c r="G46" s="400"/>
+      <c r="H46" s="400"/>
       <c r="I46" s="290"/>
       <c r="J46" s="44"/>
       <c r="K46" s="44"/>
@@ -65052,16 +65029,16 @@
       <c r="P46" s="299"/>
     </row>
     <row r="47" spans="1:16" ht="20.100000000000001" customHeight="1">
-      <c r="A47" s="402" t="s">
+      <c r="A47" s="401" t="s">
         <v>663</v>
       </c>
-      <c r="B47" s="402"/>
-      <c r="C47" s="402"/>
-      <c r="D47" s="402"/>
-      <c r="E47" s="402"/>
-      <c r="F47" s="402"/>
-      <c r="G47" s="402"/>
-      <c r="H47" s="402"/>
+      <c r="B47" s="401"/>
+      <c r="C47" s="401"/>
+      <c r="D47" s="401"/>
+      <c r="E47" s="401"/>
+      <c r="F47" s="401"/>
+      <c r="G47" s="401"/>
+      <c r="H47" s="401"/>
       <c r="I47" s="304"/>
       <c r="M47" s="291"/>
       <c r="N47" s="254"/>
@@ -65084,6 +65061,11 @@
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="A47:H47"/>
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="E1:G1"/>
+    <mergeCell ref="A36:H36"/>
+    <mergeCell ref="A46:H46"/>
     <mergeCell ref="M44:P44"/>
     <mergeCell ref="M45:P45"/>
     <mergeCell ref="A38:H38"/>
@@ -65094,11 +65076,6 @@
     <mergeCell ref="A43:H43"/>
     <mergeCell ref="A44:H44"/>
     <mergeCell ref="A45:H45"/>
-    <mergeCell ref="A47:H47"/>
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="E1:G1"/>
-    <mergeCell ref="A36:H36"/>
-    <mergeCell ref="A46:H46"/>
   </mergeCells>
   <pageMargins left="0.51181102362204722" right="0.51181102362204722" top="0.74803149606299213" bottom="0.35433070866141736" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" scale="65" orientation="portrait" r:id="rId1"/>
@@ -65151,20 +65128,20 @@
       <c r="B5" s="64"/>
       <c r="C5" s="284"/>
       <c r="D5" s="284"/>
-      <c r="E5" s="365" t="s">
+      <c r="E5" s="404" t="s">
         <v>548</v>
       </c>
-      <c r="F5" s="365"/>
+      <c r="F5" s="404"/>
     </row>
     <row r="6" spans="1:6" s="44" customFormat="1" ht="15.75" customHeight="1">
       <c r="A6" s="64"/>
       <c r="B6" s="64"/>
       <c r="C6" s="284"/>
       <c r="D6" s="284"/>
-      <c r="E6" s="365" t="s">
+      <c r="E6" s="404" t="s">
         <v>549</v>
       </c>
-      <c r="F6" s="365"/>
+      <c r="F6" s="404"/>
     </row>
     <row r="7" spans="1:6">
       <c r="E7" s="37"/>
@@ -65521,15 +65498,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="IC Publication Document" ma:contentTypeID="0x01010093EC64A4C5D74F74B7FE6AC601325A36000DFFA81A7DE45640BDB679156D0A5B85005399E94A21C7CE4A8DAA3F1632774223" ma:contentTypeVersion="37" ma:contentTypeDescription="Publication Document for IC Inventory" ma:contentTypeScope="" ma:versionID="9711fdf8ab248fc7d3dc227f0ea61d1f">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="EC08415E-A315-4408-BC27-A51AC3964F15" xmlns:ns3="571813f5-a0bc-46c9-b194-e5bb5d6c3330" xmlns:ns4="http://schemas.microsoft.com/sharepoint/v3/fields" xmlns:ns5="d060a00d-7dd1-4370-aee3-7ea2541979bf" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="fe1059bcac9d1343551fd93bdd9223e2" ns1:_="" ns2:_="" ns3:_="" ns4:_="" ns5:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -65717,6 +65685,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{51D3D907-508C-434E-81E8-1C460E28073F}">
   <ds:schemaRefs>
@@ -65731,14 +65708,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6BF01CE4-6D36-495C-93DD-85BF5C36C87F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C4E3EF8E-5DE9-4E34-9678-AF56439EF99D}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -65757,4 +65726,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/internal/2005/internalDocumentation"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6BF01CE4-6D36-495C-93DD-85BF5C36C87F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>